<commit_message>
adding Scen_Base_VS.xlsx constraints back
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_bau.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_bau.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B190DA16-CCF2-463F-A397-1A3480A38BAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{372837BB-EF09-4E22-BBEB-B0127633219C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="2" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -552,7 +552,7 @@
     <t>UC_max_oil_shale_capacity</t>
   </si>
   <si>
-    <t>C02Captured</t>
+    <t>-C02Captured</t>
   </si>
 </sst>
 </file>
@@ -8430,7 +8430,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0C1758F-E590-4DA8-B461-246947AA96DE}">
-  <dimension ref="A2:G8"/>
+  <dimension ref="A2:G6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="24.08984375" bestFit="1" customWidth="1"/>
@@ -8493,11 +8493,6 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="E8">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Adding constraint for coal
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_bau.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_bau.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{372837BB-EF09-4E22-BBEB-B0127633219C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23F07D28-5C8A-47F2-A566-18C3515F9719}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="2" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -73,7 +73,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1672" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1688" uniqueCount="169">
   <si>
     <t>~TFM_INS-TS</t>
   </si>
@@ -546,13 +546,40 @@
     <t>Pset_Set</t>
   </si>
   <si>
+    <t>LimType</t>
+  </si>
+  <si>
+    <t>UC_CAP</t>
+  </si>
+  <si>
+    <t>EST</t>
+  </si>
+  <si>
     <t>UC_RHSRT~0</t>
   </si>
   <si>
+    <t>UC_Desc</t>
+  </si>
+  <si>
+    <t>UC_min_solid_2035</t>
+  </si>
+  <si>
+    <t>pp_controllable</t>
+  </si>
+  <si>
+    <t>LO</t>
+  </si>
+  <si>
+    <t>Minimum solid fuel power plants penetration</t>
+  </si>
+  <si>
     <t>UC_max_oil_shale_capacity</t>
   </si>
   <si>
-    <t>-C02Captured</t>
+    <t>Subcritical Coal,Supercritical Coal</t>
+  </si>
+  <si>
+    <t>UP</t>
   </si>
 </sst>
 </file>
@@ -8430,66 +8457,157 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0C1758F-E590-4DA8-B461-246947AA96DE}">
-  <dimension ref="A2:G6"/>
+  <dimension ref="A2:I17"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="24.08984375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="28.453125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.6328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="11.54296875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="11.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="E4" t="s">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="D5" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
         <v>155</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B6" t="s">
         <v>156</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C6" t="s">
         <v>36</v>
       </c>
-      <c r="D5" t="s">
-        <v>18</v>
-      </c>
-      <c r="E5">
+      <c r="D6" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="E6" t="s">
+        <v>157</v>
+      </c>
+      <c r="F6" t="s">
+        <v>158</v>
+      </c>
+      <c r="G6" t="s">
+        <v>159</v>
+      </c>
+      <c r="H6" t="s">
+        <v>160</v>
+      </c>
+      <c r="I6" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>166</v>
+      </c>
+      <c r="B7" t="s">
+        <v>167</v>
+      </c>
+      <c r="D7">
         <v>2030</v>
       </c>
-      <c r="F5">
+      <c r="E7" t="s">
+        <v>168</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7">
+        <v>0.28299999999999997</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="B8" t="s">
+        <v>167</v>
+      </c>
+      <c r="D8">
         <v>2050</v>
       </c>
-      <c r="G5" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>158</v>
-      </c>
-      <c r="C6" t="s">
-        <v>78</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="E6">
-        <v>0.28299999999999997</v>
-      </c>
-      <c r="F6">
+      <c r="E8" t="s">
+        <v>168</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
+      </c>
+      <c r="G8">
         <v>0</v>
       </c>
-      <c r="G6">
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="B9" t="s">
+        <v>167</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9" t="s">
+        <v>168</v>
+      </c>
+      <c r="G9">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>162</v>
+      </c>
+      <c r="B15" t="s">
+        <v>163</v>
+      </c>
+      <c r="D15">
+        <v>2030</v>
+      </c>
+      <c r="E15" t="s">
+        <v>164</v>
+      </c>
+      <c r="F15">
+        <v>1</v>
+      </c>
+      <c r="G15">
+        <v>2</v>
+      </c>
+      <c r="I15" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="B16" t="s">
+        <v>163</v>
+      </c>
+      <c r="D16">
+        <v>2035</v>
+      </c>
+      <c r="E16" t="s">
+        <v>164</v>
+      </c>
+      <c r="F16">
+        <v>1</v>
+      </c>
+      <c r="G16">
+        <v>2.1</v>
+      </c>
+    </row>
+    <row r="17" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B17" t="s">
+        <v>163</v>
+      </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17" t="s">
+        <v>164</v>
+      </c>
+      <c r="G17">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Adding aggregation of wind and solar
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_bau.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_bau.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBBEB4F8-FA58-4224-BA9B-AFCBDE6573F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FDA0746-5C4E-4503-8F1B-4407E8791950}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -73,7 +73,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9896" uniqueCount="266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9909" uniqueCount="274">
   <si>
     <t>~TFM_INS-TS</t>
   </si>
@@ -872,6 +872,30 @@
   <si>
     <t>Keskmine kokku</t>
   </si>
+  <si>
+    <t>~UC_T: FX</t>
+  </si>
+  <si>
+    <t>pset_pn</t>
+  </si>
+  <si>
+    <t>UCE_Solar capacity aggregation for peak</t>
+  </si>
+  <si>
+    <t>ElcAgg_Solar</t>
+  </si>
+  <si>
+    <t>UCE_Wind capacity aggregation for peak</t>
+  </si>
+  <si>
+    <t>ElcAgg_Wind</t>
+  </si>
+  <si>
+    <t>wind*</t>
+  </si>
+  <si>
+    <t>*aggregate solar and wind</t>
+  </si>
 </sst>
 </file>
 
@@ -43570,15 +43594,20 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28A318F2-D986-4B43-9E10-D5047049B529}">
-  <dimension ref="A3:C5"/>
+  <dimension ref="A3:F13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="37.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -43589,7 +43618,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>102</v>
       </c>
@@ -43598,6 +43627,75 @@
       </c>
       <c r="C5" t="s">
         <v>103</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="D8" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>124</v>
+      </c>
+      <c r="B9" t="s">
+        <v>267</v>
+      </c>
+      <c r="C9" t="s">
+        <v>35</v>
+      </c>
+      <c r="D9" t="s">
+        <v>127</v>
+      </c>
+      <c r="E9" t="s">
+        <v>129</v>
+      </c>
+      <c r="F9" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>268</v>
+      </c>
+      <c r="B10" t="s">
+        <v>269</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C11" t="s">
+        <v>91</v>
+      </c>
+      <c r="D11">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>270</v>
+      </c>
+      <c r="B12" t="s">
+        <v>271</v>
+      </c>
+      <c r="D12">
+        <v>1</v>
+      </c>
+      <c r="E12">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C13" t="s">
+        <v>272</v>
+      </c>
+      <c r="D13">
+        <v>-1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Boundary on no new investements in 2025
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_bau.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_bau.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14B19A1B-38D2-4818-A3A1-6EBC4EB639F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C94E523-7404-41AE-ADE8-B7E64ED56F1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Demand" sheetId="1" r:id="rId1"/>
@@ -73,7 +73,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9909" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9914" uniqueCount="275">
   <si>
     <t>~TFM_INS-TS</t>
   </si>
@@ -893,6 +893,12 @@
   <si>
     <t>wind*</t>
   </si>
+  <si>
+    <t>ncap_bnd</t>
+  </si>
+  <si>
+    <t>year</t>
+  </si>
 </sst>
 </file>
 
@@ -44245,7 +44251,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0C1758F-E590-4DA8-B461-246947AA96DE}">
-  <dimension ref="A2:I16"/>
+  <dimension ref="A2:I21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.140625" bestFit="1" customWidth="1"/>
@@ -44382,6 +44388,33 @@
         <v>3</v>
       </c>
     </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>2</v>
+      </c>
+      <c r="B20" t="s">
+        <v>274</v>
+      </c>
+      <c r="C20" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>273</v>
+      </c>
+      <c r="B21">
+        <v>2025</v>
+      </c>
+      <c r="C21">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Remvoing boundary of 2025
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_bau.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_bau.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C94E523-7404-41AE-ADE8-B7E64ED56F1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1C8FD6D-A271-43E4-8222-E40F913C06E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -73,7 +73,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9914" uniqueCount="275">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9909" uniqueCount="273">
   <si>
     <t>~TFM_INS-TS</t>
   </si>
@@ -893,12 +893,6 @@
   <si>
     <t>wind*</t>
   </si>
-  <si>
-    <t>ncap_bnd</t>
-  </si>
-  <si>
-    <t>year</t>
-  </si>
 </sst>
 </file>
 
@@ -44251,7 +44245,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0C1758F-E590-4DA8-B461-246947AA96DE}">
-  <dimension ref="A2:I21"/>
+  <dimension ref="A2:I16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.140625" bestFit="1" customWidth="1"/>
@@ -44388,33 +44382,6 @@
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>2</v>
-      </c>
-      <c r="B20" t="s">
-        <v>274</v>
-      </c>
-      <c r="C20" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>273</v>
-      </c>
-      <c r="B21">
-        <v>2025</v>
-      </c>
-      <c r="C21">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
add 2022 trade as well
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_bau.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_bau.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB5A8D6A-91DC-41B5-AF3D-BFDCEAD96E6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EFB340A-985A-4613-B240-E711949E6C68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43707,139 +43707,142 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F0573AE-84FA-4F18-8D18-B7F3EC5B3273}">
-  <dimension ref="B4:U14"/>
+  <dimension ref="B4:V14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="20.42578125" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="43.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="2:21" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="2:21" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>11</v>
       </c>
       <c r="C5">
+        <v>2022</v>
+      </c>
+      <c r="D5">
         <v>2025</v>
       </c>
-      <c r="D5">
+      <c r="E5">
         <v>2030</v>
       </c>
-      <c r="E5">
+      <c r="F5">
         <v>2035</v>
       </c>
-      <c r="F5">
+      <c r="G5">
         <v>2040</v>
       </c>
-      <c r="G5">
+      <c r="H5">
         <v>2045</v>
       </c>
-      <c r="H5">
+      <c r="I5">
         <v>2050</v>
       </c>
-      <c r="I5" t="s">
+      <c r="J5" t="s">
         <v>2</v>
       </c>
-      <c r="J5" t="s">
+      <c r="K5" t="s">
         <v>12</v>
       </c>
-      <c r="P5" t="s">
+      <c r="Q5" t="s">
         <v>254</v>
       </c>
-      <c r="Q5" t="s">
+      <c r="R5" t="s">
         <v>255</v>
       </c>
-      <c r="R5" t="s">
+      <c r="S5" t="s">
         <v>256</v>
       </c>
-      <c r="S5" t="s">
+      <c r="T5" t="s">
         <v>257</v>
       </c>
-      <c r="T5" t="s">
+      <c r="U5" t="s">
         <v>258</v>
       </c>
-      <c r="U5" t="s">
+      <c r="V5" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="6" spans="2:21" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>13</v>
       </c>
       <c r="C6">
         <v>7.18</v>
       </c>
-      <c r="I6" t="s">
+      <c r="J6" t="s">
         <v>14</v>
       </c>
-      <c r="J6" t="s">
+      <c r="K6" t="s">
         <v>15</v>
       </c>
-      <c r="P6" t="s">
+      <c r="Q6" t="s">
         <v>260</v>
       </c>
-      <c r="Q6">
+      <c r="R6">
         <v>1147</v>
       </c>
-      <c r="R6">
+      <c r="S6">
         <v>1259</v>
       </c>
-      <c r="S6">
+      <c r="T6">
         <v>1016</v>
       </c>
-      <c r="T6">
-        <v>0</v>
-      </c>
       <c r="U6">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="V6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>16</v>
       </c>
       <c r="C7">
         <v>6.17</v>
       </c>
-      <c r="I7" t="s">
+      <c r="J7" t="s">
         <v>14</v>
       </c>
-      <c r="J7" t="s">
+      <c r="K7" t="s">
         <v>15</v>
       </c>
-      <c r="P7" t="s">
+      <c r="Q7" t="s">
         <v>261</v>
       </c>
-      <c r="Q7">
+      <c r="R7">
         <v>850</v>
       </c>
-      <c r="R7">
+      <c r="S7">
         <v>1149</v>
       </c>
-      <c r="S7">
+      <c r="T7">
         <v>1016</v>
       </c>
-      <c r="T7">
-        <v>0</v>
-      </c>
       <c r="U7">
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="2:21" x14ac:dyDescent="0.25">
+      <c r="V7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="2:22" x14ac:dyDescent="0.25">
       <c r="Q8" t="s">
         <v>262</v>
       </c>
       <c r="R8">
-        <f>SUM(Q6:Q7)/COUNT(Q6:Q7)</f>
+        <f>SUM(R6:R7)/COUNT(R6:R7)</f>
         <v>998.5</v>
       </c>
       <c r="S8">
-        <f t="shared" ref="S8:T8" si="0">SUM(R6:R7)/COUNT(R6:R7)</f>
+        <f t="shared" ref="S8:T8" si="0">SUM(S6:S7)/COUNT(S6:S7)</f>
         <v>1204</v>
       </c>
       <c r="T8">
@@ -43847,7 +43850,7 @@
         <v>1016</v>
       </c>
     </row>
-    <row r="9" spans="2:21" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:22" x14ac:dyDescent="0.25">
       <c r="Q9" t="s">
         <v>264</v>
       </c>
@@ -43856,12 +43859,12 @@
         <v>3218.5</v>
       </c>
     </row>
-    <row r="11" spans="2:21" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="2:21" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>11</v>
       </c>
@@ -43869,19 +43872,22 @@
         <v>12</v>
       </c>
       <c r="D12">
+        <v>2022</v>
+      </c>
+      <c r="E12">
         <v>2025</v>
       </c>
-      <c r="E12">
+      <c r="F12">
         <v>2030</v>
       </c>
-      <c r="F12">
+      <c r="G12">
         <v>2040</v>
       </c>
-      <c r="G12" t="s">
+      <c r="H12" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="2:21" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>16</v>
       </c>
@@ -43897,14 +43903,17 @@
       <c r="F13">
         <v>0.32185000000000002</v>
       </c>
-      <c r="G13" t="s">
+      <c r="G13">
+        <v>0.32185000000000002</v>
+      </c>
+      <c r="H13" t="s">
         <v>24</v>
       </c>
-      <c r="H13" t="s">
+      <c r="I13" t="s">
         <v>263</v>
       </c>
     </row>
-    <row r="14" spans="2:21" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>13</v>
       </c>
@@ -43920,7 +43929,10 @@
       <c r="F14">
         <v>0</v>
       </c>
-      <c r="G14" t="s">
+      <c r="G14">
+        <v>0</v>
+      </c>
+      <c r="H14" t="s">
         <v>24</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updating trades - adding CAP2ACT
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_bau.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_bau.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEED74BA-FC04-4985-8D47-B0AFE8FFA25D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D1F87DB-9AFF-4FE8-BCD7-C941AFC48C0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-80" yWindow="-80" windowWidth="19360" windowHeight="11440" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Demand" sheetId="1" r:id="rId1"/>
@@ -73,7 +73,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9927" uniqueCount="278">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9935" uniqueCount="280">
   <si>
     <t>~TFM_INS-TS</t>
   </si>
@@ -908,6 +908,12 @@
   <si>
     <t>TFM_INS-TS</t>
   </si>
+  <si>
+    <t>Trd_electricity import_ru</t>
+  </si>
+  <si>
+    <t>Trd_electricity export_ru</t>
+  </si>
 </sst>
 </file>
 
@@ -43781,19 +43787,22 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F0573AE-84FA-4F18-8D18-B7F3EC5B3273}">
-  <dimension ref="B4:V16"/>
+  <dimension ref="B4:Y18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="23.140625" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="43.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>277</v>
       </c>
-    </row>
-    <row r="5" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="X4">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="5" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>11</v>
       </c>
@@ -43842,8 +43851,14 @@
       <c r="V5" t="s">
         <v>255</v>
       </c>
-    </row>
-    <row r="6" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="X5" t="s">
+        <v>254</v>
+      </c>
+      <c r="Y5" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="6" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>272</v>
       </c>
@@ -43877,8 +43892,14 @@
       <c r="V6">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="X6">
+        <v>910</v>
+      </c>
+      <c r="Y6">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="7" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>273</v>
       </c>
@@ -43912,8 +43933,14 @@
       <c r="V7">
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="X7">
+        <v>350</v>
+      </c>
+      <c r="Y7">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="8" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>274</v>
       </c>
@@ -43937,15 +43964,31 @@
         <v>998.5</v>
       </c>
       <c r="S8">
-        <f t="shared" ref="S8:T8" si="0">SUM(S6:S7)/COUNT(S6:S7)</f>
+        <f t="shared" ref="S8:Y8" si="0">SUM(S6:S7)/COUNT(S6:S7)</f>
         <v>1204</v>
       </c>
       <c r="T8">
         <f t="shared" si="0"/>
         <v>1016</v>
       </c>
-    </row>
-    <row r="9" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="U8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="V8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="X8">
+        <f t="shared" si="0"/>
+        <v>630</v>
+      </c>
+      <c r="Y8">
+        <f t="shared" si="0"/>
+        <v>635</v>
+      </c>
+    </row>
+    <row r="9" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>275</v>
       </c>
@@ -43969,12 +44012,12 @@
         <v>3218.5</v>
       </c>
     </row>
-    <row r="11" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="12" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
         <v>11</v>
       </c>
@@ -43997,7 +44040,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
         <v>272</v>
       </c>
@@ -44027,7 +44070,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="14" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
         <v>273</v>
       </c>
@@ -44039,7 +44082,7 @@
         <v>1.204</v>
       </c>
       <c r="E14">
-        <f t="shared" ref="E14:G14" si="2">$S$8/1000</f>
+        <f t="shared" ref="E14:G15" si="2">$S$8/1000</f>
         <v>1.204</v>
       </c>
       <c r="F14">
@@ -44054,57 +44097,103 @@
         <v>20</v>
       </c>
     </row>
-    <row r="15" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:25" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
-        <v>274</v>
+        <v>278</v>
       </c>
       <c r="C15" t="s">
         <v>276</v>
       </c>
       <c r="D15">
+        <v>0.63500000000000001</v>
+      </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
+      <c r="F15">
+        <v>0</v>
+      </c>
+      <c r="G15">
+        <v>0</v>
+      </c>
+      <c r="H15" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="2:25" x14ac:dyDescent="0.25">
+      <c r="B16" t="s">
+        <v>274</v>
+      </c>
+      <c r="C16" t="s">
+        <v>276</v>
+      </c>
+      <c r="D16">
         <f>$T$6/1000</f>
         <v>1.016</v>
       </c>
-      <c r="E15">
-        <f t="shared" ref="E15:G15" si="3">$T$6/1000</f>
+      <c r="E16">
+        <f t="shared" ref="E16:G16" si="3">$T$6/1000</f>
         <v>1.016</v>
       </c>
-      <c r="F15">
+      <c r="F16">
         <f t="shared" si="3"/>
         <v>1.016</v>
       </c>
-      <c r="G15">
+      <c r="G16">
         <f t="shared" si="3"/>
         <v>1.016</v>
       </c>
-      <c r="H15" t="s">
+      <c r="H16" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="16" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B16" t="s">
+    <row r="17" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B17" t="s">
         <v>275</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C17" t="s">
         <v>276</v>
       </c>
-      <c r="D16">
+      <c r="D17">
         <f>$R$8/1000</f>
         <v>0.99850000000000005</v>
       </c>
-      <c r="E16">
-        <f t="shared" ref="E16:G16" si="4">$R$8/1000</f>
+      <c r="E17">
+        <f t="shared" ref="E17:G18" si="4">$R$8/1000</f>
         <v>0.99850000000000005</v>
       </c>
-      <c r="F16">
+      <c r="F17">
         <f t="shared" si="4"/>
         <v>0.99850000000000005</v>
       </c>
-      <c r="G16">
+      <c r="G17">
         <f t="shared" si="4"/>
         <v>0.99850000000000005</v>
       </c>
-      <c r="H16" t="s">
+      <c r="H17" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="18" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B18" t="s">
+        <v>279</v>
+      </c>
+      <c r="C18" t="s">
+        <v>276</v>
+      </c>
+      <c r="D18">
+        <v>0.63</v>
+      </c>
+      <c r="E18">
+        <v>0</v>
+      </c>
+      <c r="F18">
+        <v>0</v>
+      </c>
+      <c r="G18">
+        <v>0</v>
+      </c>
+      <c r="H18" t="s">
         <v>20</v>
       </c>
     </row>

</xml_diff>

<commit_message>
restrict import from finland
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_bau.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_bau.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C7EAA00-52F5-4FFE-B832-20E21232147A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78294755-A798-438E-8A18-62F814A76FDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Demand" sheetId="1" r:id="rId1"/>
@@ -43969,6 +43969,9 @@
       <c r="H7">
         <v>0</v>
       </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
       <c r="J7" t="s">
         <v>13</v>
       </c>

</xml_diff>

<commit_message>
setting mimimum export to lv
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_bau.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_bau.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78294755-A798-438E-8A18-62F814A76FDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98A387F6-67F8-47ED-A0FC-3ED57372EE09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44061,6 +44061,21 @@
       <c r="D9">
         <v>1.64</v>
       </c>
+      <c r="E9">
+        <v>1.64</v>
+      </c>
+      <c r="F9">
+        <v>1.64</v>
+      </c>
+      <c r="G9">
+        <v>1.64</v>
+      </c>
+      <c r="H9">
+        <v>1.64</v>
+      </c>
+      <c r="I9">
+        <v>1.64</v>
+      </c>
       <c r="J9" t="s">
         <v>13</v>
       </c>

</xml_diff>

<commit_message>
setting maximum import from finland
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_bau.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_bau.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98A387F6-67F8-47ED-A0FC-3ED57372EE09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC093415-0638-4CAF-A794-A8C22FBA62C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43846,6 +43846,9 @@
       <c r="B4" t="s">
         <v>0</v>
       </c>
+      <c r="E4">
+        <v>0.04</v>
+      </c>
       <c r="X4">
         <v>2022</v>
       </c>
@@ -43916,11 +43919,31 @@
       <c r="D6">
         <v>4.68</v>
       </c>
+      <c r="E6">
+        <f>D6-(D6*$E$4)</f>
+        <v>4.4927999999999999</v>
+      </c>
+      <c r="F6">
+        <f t="shared" ref="F6:I6" si="0">E6-(E6*$E$4)</f>
+        <v>4.3130879999999996</v>
+      </c>
+      <c r="G6">
+        <f t="shared" si="0"/>
+        <v>4.1405644799999992</v>
+      </c>
+      <c r="H6">
+        <f t="shared" si="0"/>
+        <v>3.9749419007999993</v>
+      </c>
+      <c r="I6">
+        <f t="shared" si="0"/>
+        <v>3.8159442247679993</v>
+      </c>
       <c r="J6" t="s">
         <v>13</v>
       </c>
       <c r="K6" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="Q6" t="s">
         <v>254</v>
@@ -44027,27 +44050,27 @@
         <v>998.5</v>
       </c>
       <c r="S8">
-        <f t="shared" ref="S8:Y8" si="0">SUM(S6:S7)/COUNT(S6:S7)</f>
+        <f t="shared" ref="S8:Y8" si="1">SUM(S6:S7)/COUNT(S6:S7)</f>
         <v>1204</v>
       </c>
       <c r="T8">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1016</v>
       </c>
       <c r="U8">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="V8">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="X8">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>630</v>
       </c>
       <c r="Y8">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>635</v>
       </c>
     </row>
@@ -44136,23 +44159,23 @@
         <v>1.016</v>
       </c>
       <c r="E13">
-        <f t="shared" ref="E13:I13" si="1">$T$6/1000</f>
+        <f t="shared" ref="E13:I13" si="2">$T$6/1000</f>
         <v>1.016</v>
       </c>
       <c r="F13">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1.016</v>
       </c>
       <c r="G13">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1.016</v>
       </c>
       <c r="H13">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1.016</v>
       </c>
       <c r="I13">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1.016</v>
       </c>
       <c r="J13" t="s">
@@ -44174,23 +44197,23 @@
         <v>1.204</v>
       </c>
       <c r="E14">
-        <f t="shared" ref="E14:I14" si="2">$S$8/1000</f>
+        <f t="shared" ref="E14:I14" si="3">$S$8/1000</f>
         <v>1.204</v>
       </c>
       <c r="F14">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.204</v>
       </c>
       <c r="G14">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.204</v>
       </c>
       <c r="H14">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.204</v>
       </c>
       <c r="I14">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.204</v>
       </c>
       <c r="J14" t="s">
@@ -44209,23 +44232,23 @@
         <v>1.016</v>
       </c>
       <c r="E15">
-        <f t="shared" ref="E15:I15" si="3">$T$6/1000</f>
+        <f t="shared" ref="E15:I15" si="4">$T$6/1000</f>
         <v>1.016</v>
       </c>
       <c r="F15">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1.016</v>
       </c>
       <c r="G15">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1.016</v>
       </c>
       <c r="H15">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1.016</v>
       </c>
       <c r="I15">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1.016</v>
       </c>
       <c r="J15" t="s">
@@ -44244,23 +44267,23 @@
         <v>0.99850000000000005</v>
       </c>
       <c r="E16">
-        <f t="shared" ref="E16:I16" si="4">$R$8/1000</f>
+        <f t="shared" ref="E16:I16" si="5">$R$8/1000</f>
         <v>0.99850000000000005</v>
       </c>
       <c r="F16">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0.99850000000000005</v>
       </c>
       <c r="G16">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0.99850000000000005</v>
       </c>
       <c r="H16">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0.99850000000000005</v>
       </c>
       <c r="I16">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>0.99850000000000005</v>
       </c>
       <c r="J16" t="s">

</xml_diff>

<commit_message>
Adding timesliced ncap_afc to trd electricity import from finland
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_bau.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_bau.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB5F7983-B2B0-49C9-8A31-BAB9DE9B3327}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBB83B1D-AEBC-4C9C-ADF0-A3952AE3607A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-10470" yWindow="10890" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Demand" sheetId="1" r:id="rId1"/>
@@ -73,7 +73,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6213" uniqueCount="284">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6506" uniqueCount="287">
   <si>
     <t>~TFM_INS-TS</t>
   </si>
@@ -926,6 +926,15 @@
   <si>
     <t>TFM_DINS-AT</t>
   </si>
+  <si>
+    <t>Timeslice</t>
+  </si>
+  <si>
+    <t>Attribute</t>
+  </si>
+  <si>
+    <t>NCAP_AFC</t>
+  </si>
 </sst>
 </file>
 
@@ -1029,21 +1038,21 @@
     </sheetNames>
     <sheetDataSet>
       <sheetData sheetId="0"/>
-      <sheetData sheetId="1" refreshError="1"/>
-      <sheetData sheetId="2" refreshError="1"/>
-      <sheetData sheetId="3" refreshError="1"/>
-      <sheetData sheetId="4" refreshError="1"/>
-      <sheetData sheetId="5" refreshError="1"/>
-      <sheetData sheetId="6" refreshError="1"/>
-      <sheetData sheetId="7" refreshError="1"/>
-      <sheetData sheetId="8" refreshError="1"/>
-      <sheetData sheetId="9" refreshError="1"/>
-      <sheetData sheetId="10" refreshError="1"/>
-      <sheetData sheetId="11" refreshError="1"/>
-      <sheetData sheetId="12" refreshError="1"/>
-      <sheetData sheetId="13" refreshError="1"/>
-      <sheetData sheetId="14" refreshError="1"/>
-      <sheetData sheetId="15" refreshError="1"/>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4"/>
+      <sheetData sheetId="5"/>
+      <sheetData sheetId="6"/>
+      <sheetData sheetId="7"/>
+      <sheetData sheetId="8"/>
+      <sheetData sheetId="9"/>
+      <sheetData sheetId="10"/>
+      <sheetData sheetId="11"/>
+      <sheetData sheetId="12"/>
+      <sheetData sheetId="13"/>
+      <sheetData sheetId="14"/>
+      <sheetData sheetId="15"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -1747,7 +1756,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05B64E1E-DC66-450D-AA2A-D1B01A72BCA4}">
-  <dimension ref="A1:AN962"/>
+  <dimension ref="A1:AW962"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="6" max="6" width="44.42578125" bestFit="1" customWidth="1"/>
@@ -1764,9 +1773,13 @@
     <col min="36" max="36" width="14.140625" bestFit="1" customWidth="1"/>
     <col min="38" max="38" width="14.140625" bestFit="1" customWidth="1"/>
     <col min="40" max="40" width="12" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="22.85546875" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="9.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:40" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:48" x14ac:dyDescent="0.25">
       <c r="C1" t="s">
         <v>49</v>
       </c>
@@ -1791,8 +1804,11 @@
       <c r="AK1" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="2" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="AQ1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2" spans="1:48" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>48</v>
       </c>
@@ -1889,8 +1905,20 @@
       <c r="AN2" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="AQ2" t="s">
+        <v>284</v>
+      </c>
+      <c r="AR2" t="s">
+        <v>285</v>
+      </c>
+      <c r="AS2" t="s">
+        <v>11</v>
+      </c>
+      <c r="AT2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:48" x14ac:dyDescent="0.25">
       <c r="A3" t="str">
         <f>IFERROR(IF([1]Veda!#REF!=A2,"ok","x"),"")</f>
         <v/>
@@ -1988,8 +2016,24 @@
       <c r="AN3" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="4" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="AQ3" t="s">
+        <v>122</v>
+      </c>
+      <c r="AR3" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS3" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT3">
+        <f>350/$AV$3</f>
+        <v>0.34448818897637795</v>
+      </c>
+      <c r="AV3">
+        <v>1016</v>
+      </c>
+    </row>
+    <row r="4" spans="1:48" x14ac:dyDescent="0.25">
       <c r="C4" t="s">
         <v>104</v>
       </c>
@@ -2077,8 +2121,21 @@
       <c r="AN4" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="5" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="AQ4" t="s">
+        <v>123</v>
+      </c>
+      <c r="AR4" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS4" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT4">
+        <f t="shared" ref="AT4:AT24" si="0">350/$AV$3</f>
+        <v>0.34448818897637795</v>
+      </c>
+    </row>
+    <row r="5" spans="1:48" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
         <v>106</v>
       </c>
@@ -2166,8 +2223,21 @@
       <c r="AN5" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="6" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="AQ5" t="s">
+        <v>124</v>
+      </c>
+      <c r="AR5" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS5" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT5">
+        <f t="shared" si="0"/>
+        <v>0.34448818897637795</v>
+      </c>
+    </row>
+    <row r="6" spans="1:48" x14ac:dyDescent="0.25">
       <c r="C6" t="s">
         <v>108</v>
       </c>
@@ -2255,8 +2325,21 @@
       <c r="AN6" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="7" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="AQ6" t="s">
+        <v>125</v>
+      </c>
+      <c r="AR6" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS6" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT6">
+        <f t="shared" si="0"/>
+        <v>0.34448818897637795</v>
+      </c>
+    </row>
+    <row r="7" spans="1:48" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
         <v>110</v>
       </c>
@@ -2344,8 +2427,21 @@
       <c r="AN7" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="8" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="AQ7" t="s">
+        <v>126</v>
+      </c>
+      <c r="AR7" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS7" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT7">
+        <f t="shared" si="0"/>
+        <v>0.34448818897637795</v>
+      </c>
+    </row>
+    <row r="8" spans="1:48" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
         <v>112</v>
       </c>
@@ -2433,8 +2529,21 @@
       <c r="AN8" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="9" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="AQ8" t="s">
+        <v>127</v>
+      </c>
+      <c r="AR8" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS8" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT8">
+        <f t="shared" si="0"/>
+        <v>0.34448818897637795</v>
+      </c>
+    </row>
+    <row r="9" spans="1:48" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
         <v>114</v>
       </c>
@@ -2522,8 +2631,21 @@
       <c r="AN9" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="10" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="AQ9" t="s">
+        <v>128</v>
+      </c>
+      <c r="AR9" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS9" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT9">
+        <f t="shared" si="0"/>
+        <v>0.34448818897637795</v>
+      </c>
+    </row>
+    <row r="10" spans="1:48" x14ac:dyDescent="0.25">
       <c r="C10" t="s">
         <v>116</v>
       </c>
@@ -2611,8 +2733,21 @@
       <c r="AN10" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="11" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="AQ10" t="s">
+        <v>129</v>
+      </c>
+      <c r="AR10" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS10" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT10">
+        <f t="shared" si="0"/>
+        <v>0.34448818897637795</v>
+      </c>
+    </row>
+    <row r="11" spans="1:48" x14ac:dyDescent="0.25">
       <c r="C11" t="s">
         <v>118</v>
       </c>
@@ -2694,8 +2829,21 @@
       <c r="AN11" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="12" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="AQ11" t="s">
+        <v>130</v>
+      </c>
+      <c r="AR11" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS11" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT11">
+        <f t="shared" si="0"/>
+        <v>0.34448818897637795</v>
+      </c>
+    </row>
+    <row r="12" spans="1:48" x14ac:dyDescent="0.25">
       <c r="C12" t="s">
         <v>119</v>
       </c>
@@ -2777,8 +2925,21 @@
       <c r="AN12" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="13" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="AQ12" t="s">
+        <v>131</v>
+      </c>
+      <c r="AR12" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS12" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT12">
+        <f t="shared" si="0"/>
+        <v>0.34448818897637795</v>
+      </c>
+    </row>
+    <row r="13" spans="1:48" x14ac:dyDescent="0.25">
       <c r="C13" t="s">
         <v>120</v>
       </c>
@@ -2860,8 +3021,21 @@
       <c r="AN13" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="14" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="AQ13" t="s">
+        <v>132</v>
+      </c>
+      <c r="AR13" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS13" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT13">
+        <f t="shared" si="0"/>
+        <v>0.34448818897637795</v>
+      </c>
+    </row>
+    <row r="14" spans="1:48" x14ac:dyDescent="0.25">
       <c r="C14" t="s">
         <v>121</v>
       </c>
@@ -2943,8 +3117,21 @@
       <c r="AN14" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="15" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="AQ14" t="s">
+        <v>133</v>
+      </c>
+      <c r="AR14" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS14" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT14">
+        <f t="shared" si="0"/>
+        <v>0.34448818897637795</v>
+      </c>
+    </row>
+    <row r="15" spans="1:48" x14ac:dyDescent="0.25">
       <c r="I15" t="s">
         <v>266</v>
       </c>
@@ -3023,8 +3210,21 @@
       <c r="AN15" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="16" spans="1:40" x14ac:dyDescent="0.25">
+      <c r="AQ15" t="s">
+        <v>134</v>
+      </c>
+      <c r="AR15" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS15" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT15">
+        <f t="shared" si="0"/>
+        <v>0.34448818897637795</v>
+      </c>
+    </row>
+    <row r="16" spans="1:48" x14ac:dyDescent="0.25">
       <c r="I16" t="s">
         <v>266</v>
       </c>
@@ -3103,8 +3303,21 @@
       <c r="AN16" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="17" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ16" t="s">
+        <v>135</v>
+      </c>
+      <c r="AR16" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS16" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT16">
+        <f t="shared" si="0"/>
+        <v>0.34448818897637795</v>
+      </c>
+    </row>
+    <row r="17" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I17" t="s">
         <v>266</v>
       </c>
@@ -3183,8 +3396,21 @@
       <c r="AN17" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="18" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ17" t="s">
+        <v>136</v>
+      </c>
+      <c r="AR17" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS17" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT17">
+        <f t="shared" si="0"/>
+        <v>0.34448818897637795</v>
+      </c>
+    </row>
+    <row r="18" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I18" t="s">
         <v>266</v>
       </c>
@@ -3263,8 +3489,21 @@
       <c r="AN18" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="19" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ18" t="s">
+        <v>137</v>
+      </c>
+      <c r="AR18" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS18" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT18">
+        <f t="shared" si="0"/>
+        <v>0.34448818897637795</v>
+      </c>
+    </row>
+    <row r="19" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I19" t="s">
         <v>266</v>
       </c>
@@ -3343,8 +3582,21 @@
       <c r="AN19" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="20" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ19" t="s">
+        <v>138</v>
+      </c>
+      <c r="AR19" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS19" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT19">
+        <f t="shared" si="0"/>
+        <v>0.34448818897637795</v>
+      </c>
+    </row>
+    <row r="20" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I20" t="s">
         <v>266</v>
       </c>
@@ -3423,8 +3675,21 @@
       <c r="AN20" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="21" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ20" t="s">
+        <v>139</v>
+      </c>
+      <c r="AR20" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS20" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT20">
+        <f t="shared" si="0"/>
+        <v>0.34448818897637795</v>
+      </c>
+    </row>
+    <row r="21" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I21" t="s">
         <v>266</v>
       </c>
@@ -3503,8 +3768,21 @@
       <c r="AN21" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="22" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ21" t="s">
+        <v>140</v>
+      </c>
+      <c r="AR21" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS21" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT21">
+        <f t="shared" si="0"/>
+        <v>0.34448818897637795</v>
+      </c>
+    </row>
+    <row r="22" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I22" t="s">
         <v>266</v>
       </c>
@@ -3583,8 +3861,21 @@
       <c r="AN22" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="23" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ22" t="s">
+        <v>141</v>
+      </c>
+      <c r="AR22" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS22" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT22">
+        <f t="shared" si="0"/>
+        <v>0.34448818897637795</v>
+      </c>
+    </row>
+    <row r="23" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I23" t="s">
         <v>266</v>
       </c>
@@ -3663,8 +3954,21 @@
       <c r="AN23" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="24" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ23" t="s">
+        <v>142</v>
+      </c>
+      <c r="AR23" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS23" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT23">
+        <f t="shared" si="0"/>
+        <v>0.34448818897637795</v>
+      </c>
+    </row>
+    <row r="24" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I24" t="s">
         <v>266</v>
       </c>
@@ -3743,8 +4047,21 @@
       <c r="AN24" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="25" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ24" t="s">
+        <v>143</v>
+      </c>
+      <c r="AR24" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS24" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT24">
+        <f t="shared" si="0"/>
+        <v>0.34448818897637795</v>
+      </c>
+    </row>
+    <row r="25" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I25" t="s">
         <v>266</v>
       </c>
@@ -3823,8 +4140,24 @@
       <c r="AN25" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="26" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ25" t="s">
+        <v>144</v>
+      </c>
+      <c r="AR25" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS25" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT25">
+        <v>0.79</v>
+      </c>
+      <c r="AW25" s="2">
+        <f ca="1">RANDBETWEEN(70,95)/100</f>
+        <v>0.76</v>
+      </c>
+    </row>
+    <row r="26" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I26" t="s">
         <v>266</v>
       </c>
@@ -3903,8 +4236,24 @@
       <c r="AN26" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="27" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ26" t="s">
+        <v>145</v>
+      </c>
+      <c r="AR26" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS26" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT26">
+        <v>0.85</v>
+      </c>
+      <c r="AW26" s="2">
+        <f t="shared" ref="AW26:AW89" ca="1" si="1">RANDBETWEEN(70,95)/100</f>
+        <v>0.72</v>
+      </c>
+    </row>
+    <row r="27" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I27" t="s">
         <v>266</v>
       </c>
@@ -3983,8 +4332,24 @@
       <c r="AN27" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="28" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ27" t="s">
+        <v>146</v>
+      </c>
+      <c r="AR27" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS27" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT27">
+        <v>0.72</v>
+      </c>
+      <c r="AW27" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.72</v>
+      </c>
+    </row>
+    <row r="28" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I28" t="s">
         <v>266</v>
       </c>
@@ -4063,8 +4428,24 @@
       <c r="AN28" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="29" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ28" t="s">
+        <v>147</v>
+      </c>
+      <c r="AR28" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS28" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT28">
+        <v>0.79</v>
+      </c>
+      <c r="AW28" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.81</v>
+      </c>
+    </row>
+    <row r="29" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I29" t="s">
         <v>266</v>
       </c>
@@ -4143,8 +4524,24 @@
       <c r="AN29" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="30" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ29" t="s">
+        <v>148</v>
+      </c>
+      <c r="AR29" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS29" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT29">
+        <v>0.83</v>
+      </c>
+      <c r="AW29" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.93</v>
+      </c>
+    </row>
+    <row r="30" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I30" t="s">
         <v>266</v>
       </c>
@@ -4223,8 +4620,24 @@
       <c r="AN30" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="31" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ30" t="s">
+        <v>149</v>
+      </c>
+      <c r="AR30" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS30" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT30">
+        <v>0.77</v>
+      </c>
+      <c r="AW30" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.79</v>
+      </c>
+    </row>
+    <row r="31" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I31" t="s">
         <v>266</v>
       </c>
@@ -4303,8 +4716,24 @@
       <c r="AN31" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="32" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ31" t="s">
+        <v>150</v>
+      </c>
+      <c r="AR31" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS31" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT31">
+        <v>0.74</v>
+      </c>
+      <c r="AW31" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.77</v>
+      </c>
+    </row>
+    <row r="32" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I32" t="s">
         <v>266</v>
       </c>
@@ -4383,8 +4812,24 @@
       <c r="AN32" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="33" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ32" t="s">
+        <v>151</v>
+      </c>
+      <c r="AR32" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS32" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT32">
+        <v>0.87</v>
+      </c>
+      <c r="AW32" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.89</v>
+      </c>
+    </row>
+    <row r="33" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I33" t="s">
         <v>266</v>
       </c>
@@ -4463,8 +4908,24 @@
       <c r="AN33" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="34" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ33" t="s">
+        <v>152</v>
+      </c>
+      <c r="AR33" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS33" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT33">
+        <v>0.71</v>
+      </c>
+      <c r="AW33" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.83</v>
+      </c>
+    </row>
+    <row r="34" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I34" t="s">
         <v>266</v>
       </c>
@@ -4543,8 +5004,24 @@
       <c r="AN34" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="35" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ34" t="s">
+        <v>153</v>
+      </c>
+      <c r="AR34" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS34" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT34">
+        <v>0.88</v>
+      </c>
+      <c r="AW34" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="35" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I35" t="s">
         <v>266</v>
       </c>
@@ -4623,8 +5100,24 @@
       <c r="AN35" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="36" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ35" t="s">
+        <v>154</v>
+      </c>
+      <c r="AR35" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS35" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT35">
+        <v>0.74</v>
+      </c>
+      <c r="AW35" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.93</v>
+      </c>
+    </row>
+    <row r="36" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I36" t="s">
         <v>266</v>
       </c>
@@ -4703,8 +5196,24 @@
       <c r="AN36" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="37" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ36" t="s">
+        <v>155</v>
+      </c>
+      <c r="AR36" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS36" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT36">
+        <v>0.92</v>
+      </c>
+      <c r="AW36" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.87</v>
+      </c>
+    </row>
+    <row r="37" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I37" t="s">
         <v>266</v>
       </c>
@@ -4783,8 +5292,24 @@
       <c r="AN37" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="38" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ37" t="s">
+        <v>156</v>
+      </c>
+      <c r="AR37" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS37" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT37">
+        <v>0.73</v>
+      </c>
+      <c r="AW37" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.71</v>
+      </c>
+    </row>
+    <row r="38" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I38" t="s">
         <v>266</v>
       </c>
@@ -4863,8 +5388,24 @@
       <c r="AN38" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="39" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ38" t="s">
+        <v>157</v>
+      </c>
+      <c r="AR38" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS38" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT38">
+        <v>0.89</v>
+      </c>
+      <c r="AW38" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.71</v>
+      </c>
+    </row>
+    <row r="39" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I39" t="s">
         <v>266</v>
       </c>
@@ -4931,8 +5472,24 @@
       <c r="AN39" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="40" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ39" t="s">
+        <v>158</v>
+      </c>
+      <c r="AR39" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS39" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT39">
+        <v>0.72</v>
+      </c>
+      <c r="AW39" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="40" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I40" t="s">
         <v>266</v>
       </c>
@@ -4999,8 +5556,24 @@
       <c r="AN40" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="41" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ40" t="s">
+        <v>159</v>
+      </c>
+      <c r="AR40" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS40" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT40">
+        <v>0.81</v>
+      </c>
+      <c r="AW40" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="41" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I41" t="s">
         <v>266</v>
       </c>
@@ -5067,8 +5640,24 @@
       <c r="AN41" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="42" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ41" t="s">
+        <v>160</v>
+      </c>
+      <c r="AR41" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS41" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT41">
+        <v>0.78</v>
+      </c>
+      <c r="AW41" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="42" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I42" t="s">
         <v>266</v>
       </c>
@@ -5135,8 +5724,24 @@
       <c r="AN42" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="43" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ42" t="s">
+        <v>161</v>
+      </c>
+      <c r="AR42" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS42" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT42">
+        <v>0.79</v>
+      </c>
+      <c r="AW42" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.84</v>
+      </c>
+    </row>
+    <row r="43" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I43" t="s">
         <v>266</v>
       </c>
@@ -5203,8 +5808,24 @@
       <c r="AN43" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="44" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ43" t="s">
+        <v>162</v>
+      </c>
+      <c r="AR43" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS43" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT43">
+        <v>0.87</v>
+      </c>
+      <c r="AW43" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.93</v>
+      </c>
+    </row>
+    <row r="44" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I44" t="s">
         <v>266</v>
       </c>
@@ -5271,8 +5892,24 @@
       <c r="AN44" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="45" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ44" t="s">
+        <v>163</v>
+      </c>
+      <c r="AR44" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS44" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT44">
+        <v>0.7</v>
+      </c>
+      <c r="AW44" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="45" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I45" t="s">
         <v>266</v>
       </c>
@@ -5339,8 +5976,24 @@
       <c r="AN45" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="46" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ45" t="s">
+        <v>164</v>
+      </c>
+      <c r="AR45" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS45" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT45">
+        <v>0.8</v>
+      </c>
+      <c r="AW45" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.82</v>
+      </c>
+    </row>
+    <row r="46" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I46" t="s">
         <v>266</v>
       </c>
@@ -5407,8 +6060,24 @@
       <c r="AN46" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="47" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ46" t="s">
+        <v>165</v>
+      </c>
+      <c r="AR46" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS46" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT46">
+        <v>0.95</v>
+      </c>
+      <c r="AW46" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.88</v>
+      </c>
+    </row>
+    <row r="47" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I47" t="s">
         <v>266</v>
       </c>
@@ -5475,8 +6144,24 @@
       <c r="AN47" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="48" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ47" t="s">
+        <v>166</v>
+      </c>
+      <c r="AR47" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS47" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT47">
+        <v>0.87</v>
+      </c>
+      <c r="AW47" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.89</v>
+      </c>
+    </row>
+    <row r="48" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I48" t="s">
         <v>266</v>
       </c>
@@ -5543,8 +6228,24 @@
       <c r="AN48" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="49" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ48" t="s">
+        <v>167</v>
+      </c>
+      <c r="AR48" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS48" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT48">
+        <v>0.84</v>
+      </c>
+      <c r="AW48" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.78</v>
+      </c>
+    </row>
+    <row r="49" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I49" t="s">
         <v>266</v>
       </c>
@@ -5611,8 +6312,24 @@
       <c r="AN49" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="50" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ49" t="s">
+        <v>168</v>
+      </c>
+      <c r="AR49" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS49" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT49">
+        <v>0.74</v>
+      </c>
+      <c r="AW49" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.72</v>
+      </c>
+    </row>
+    <row r="50" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I50" t="s">
         <v>266</v>
       </c>
@@ -5679,8 +6396,24 @@
       <c r="AN50" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="51" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ50" t="s">
+        <v>169</v>
+      </c>
+      <c r="AR50" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS50" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT50">
+        <v>0.89</v>
+      </c>
+      <c r="AW50" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.72</v>
+      </c>
+    </row>
+    <row r="51" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I51" t="s">
         <v>266</v>
       </c>
@@ -5747,8 +6480,24 @@
       <c r="AN51" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="52" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ51" t="s">
+        <v>170</v>
+      </c>
+      <c r="AR51" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS51" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT51">
+        <v>0.73</v>
+      </c>
+      <c r="AW51" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.87</v>
+      </c>
+    </row>
+    <row r="52" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I52" t="s">
         <v>266</v>
       </c>
@@ -5815,8 +6564,24 @@
       <c r="AN52" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="53" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ52" t="s">
+        <v>171</v>
+      </c>
+      <c r="AR52" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS52" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT52">
+        <v>0.91</v>
+      </c>
+      <c r="AW52" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.74</v>
+      </c>
+    </row>
+    <row r="53" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I53" t="s">
         <v>266</v>
       </c>
@@ -5883,8 +6648,24 @@
       <c r="AN53" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="54" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ53" t="s">
+        <v>172</v>
+      </c>
+      <c r="AR53" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS53" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT53">
+        <v>0.9</v>
+      </c>
+      <c r="AW53" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.78</v>
+      </c>
+    </row>
+    <row r="54" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I54" t="s">
         <v>266</v>
       </c>
@@ -5951,8 +6732,24 @@
       <c r="AN54" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="55" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ54" t="s">
+        <v>173</v>
+      </c>
+      <c r="AR54" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS54" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT54">
+        <v>0.88</v>
+      </c>
+      <c r="AW54" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="55" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I55" t="s">
         <v>266</v>
       </c>
@@ -6019,8 +6816,24 @@
       <c r="AN55" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="56" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ55" t="s">
+        <v>174</v>
+      </c>
+      <c r="AR55" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS55" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT55">
+        <v>0.78</v>
+      </c>
+      <c r="AW55" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.79</v>
+      </c>
+    </row>
+    <row r="56" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I56" t="s">
         <v>266</v>
       </c>
@@ -6087,8 +6900,24 @@
       <c r="AN56" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="57" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ56" t="s">
+        <v>175</v>
+      </c>
+      <c r="AR56" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS56" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT56">
+        <v>0.78</v>
+      </c>
+      <c r="AW56" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.88</v>
+      </c>
+    </row>
+    <row r="57" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I57" t="s">
         <v>266</v>
       </c>
@@ -6155,8 +6984,24 @@
       <c r="AN57" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="58" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ57" t="s">
+        <v>176</v>
+      </c>
+      <c r="AR57" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS57" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT57">
+        <v>0.8</v>
+      </c>
+      <c r="AW57" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="58" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I58" t="s">
         <v>266</v>
       </c>
@@ -6223,8 +7068,24 @@
       <c r="AN58" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="59" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ58" t="s">
+        <v>177</v>
+      </c>
+      <c r="AR58" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS58" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT58">
+        <v>0.7</v>
+      </c>
+      <c r="AW58" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.81</v>
+      </c>
+    </row>
+    <row r="59" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I59" t="s">
         <v>266</v>
       </c>
@@ -6291,8 +7152,24 @@
       <c r="AN59" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="60" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ59" t="s">
+        <v>178</v>
+      </c>
+      <c r="AR59" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS59" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT59">
+        <v>0.84</v>
+      </c>
+      <c r="AW59" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="60" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I60" t="s">
         <v>266</v>
       </c>
@@ -6359,8 +7236,24 @@
       <c r="AN60" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="61" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ60" t="s">
+        <v>179</v>
+      </c>
+      <c r="AR60" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS60" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT60">
+        <v>0.86</v>
+      </c>
+      <c r="AW60" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.89</v>
+      </c>
+    </row>
+    <row r="61" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I61" t="s">
         <v>266</v>
       </c>
@@ -6427,8 +7320,24 @@
       <c r="AN61" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="62" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ61" t="s">
+        <v>180</v>
+      </c>
+      <c r="AR61" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS61" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT61">
+        <v>0.92</v>
+      </c>
+      <c r="AW61" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.81</v>
+      </c>
+    </row>
+    <row r="62" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I62" t="s">
         <v>266</v>
       </c>
@@ -6495,8 +7404,24 @@
       <c r="AN62" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="63" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ62" t="s">
+        <v>181</v>
+      </c>
+      <c r="AR62" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS62" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT62">
+        <v>0.87</v>
+      </c>
+      <c r="AW62" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="63" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I63" t="s">
         <v>266</v>
       </c>
@@ -6563,8 +7488,24 @@
       <c r="AN63" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="64" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ63" t="s">
+        <v>182</v>
+      </c>
+      <c r="AR63" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS63" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT63">
+        <v>0.86</v>
+      </c>
+      <c r="AW63" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="64" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I64" t="s">
         <v>266</v>
       </c>
@@ -6631,8 +7572,24 @@
       <c r="AN64" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="65" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ64" t="s">
+        <v>183</v>
+      </c>
+      <c r="AR64" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS64" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT64">
+        <v>0.81</v>
+      </c>
+      <c r="AW64" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.94</v>
+      </c>
+    </row>
+    <row r="65" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I65" t="s">
         <v>266</v>
       </c>
@@ -6699,8 +7656,24 @@
       <c r="AN65" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="66" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ65" t="s">
+        <v>184</v>
+      </c>
+      <c r="AR65" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS65" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT65">
+        <v>0.84</v>
+      </c>
+      <c r="AW65" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="66" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I66" t="s">
         <v>266</v>
       </c>
@@ -6767,8 +7740,24 @@
       <c r="AN66" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="67" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ66" t="s">
+        <v>185</v>
+      </c>
+      <c r="AR66" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS66" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT66">
+        <v>0.8</v>
+      </c>
+      <c r="AW66" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="67" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I67" t="s">
         <v>266</v>
       </c>
@@ -6835,8 +7824,24 @@
       <c r="AN67" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="68" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ67" t="s">
+        <v>186</v>
+      </c>
+      <c r="AR67" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS67" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT67">
+        <v>0.83</v>
+      </c>
+      <c r="AW67" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.81</v>
+      </c>
+    </row>
+    <row r="68" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I68" t="s">
         <v>266</v>
       </c>
@@ -6903,8 +7908,24 @@
       <c r="AN68" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="69" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ68" t="s">
+        <v>187</v>
+      </c>
+      <c r="AR68" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS68" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT68">
+        <v>0.84</v>
+      </c>
+      <c r="AW68" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.72</v>
+      </c>
+    </row>
+    <row r="69" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I69" t="s">
         <v>266</v>
       </c>
@@ -6971,8 +7992,24 @@
       <c r="AN69" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="70" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ69" t="s">
+        <v>188</v>
+      </c>
+      <c r="AR69" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS69" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT69">
+        <v>0.78</v>
+      </c>
+      <c r="AW69" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.79</v>
+      </c>
+    </row>
+    <row r="70" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I70" t="s">
         <v>266</v>
       </c>
@@ -7039,8 +8076,24 @@
       <c r="AN70" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="71" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ70" t="s">
+        <v>189</v>
+      </c>
+      <c r="AR70" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS70" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT70">
+        <v>0.86</v>
+      </c>
+      <c r="AW70" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.82</v>
+      </c>
+    </row>
+    <row r="71" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I71" t="s">
         <v>266</v>
       </c>
@@ -7107,8 +8160,24 @@
       <c r="AN71" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="72" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ71" t="s">
+        <v>190</v>
+      </c>
+      <c r="AR71" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS71" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT71">
+        <v>0.79</v>
+      </c>
+      <c r="AW71" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.91</v>
+      </c>
+    </row>
+    <row r="72" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I72" t="s">
         <v>266</v>
       </c>
@@ -7175,8 +8244,24 @@
       <c r="AN72" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="73" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ72" t="s">
+        <v>191</v>
+      </c>
+      <c r="AR72" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS72" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT72">
+        <v>0.88</v>
+      </c>
+      <c r="AW72" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="73" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I73" t="s">
         <v>266</v>
       </c>
@@ -7243,8 +8328,24 @@
       <c r="AN73" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="74" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ73" t="s">
+        <v>192</v>
+      </c>
+      <c r="AR73" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS73" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT73">
+        <v>0.9</v>
+      </c>
+      <c r="AW73" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.87</v>
+      </c>
+    </row>
+    <row r="74" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I74" t="s">
         <v>266</v>
       </c>
@@ -7311,8 +8412,24 @@
       <c r="AN74" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="75" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ74" t="s">
+        <v>193</v>
+      </c>
+      <c r="AR74" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS74" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT74">
+        <v>0.79</v>
+      </c>
+      <c r="AW74" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.73</v>
+      </c>
+    </row>
+    <row r="75" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I75" t="s">
         <v>266</v>
       </c>
@@ -7379,8 +8496,24 @@
       <c r="AN75" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="76" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ75" t="s">
+        <v>194</v>
+      </c>
+      <c r="AR75" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS75" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT75">
+        <v>0.85</v>
+      </c>
+      <c r="AW75" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="76" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I76" t="s">
         <v>266</v>
       </c>
@@ -7447,8 +8580,24 @@
       <c r="AN76" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="77" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ76" t="s">
+        <v>195</v>
+      </c>
+      <c r="AR76" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS76" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT76">
+        <v>0.78</v>
+      </c>
+      <c r="AW76" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.76</v>
+      </c>
+    </row>
+    <row r="77" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I77" t="s">
         <v>266</v>
       </c>
@@ -7515,8 +8664,24 @@
       <c r="AN77" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="78" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ77" t="s">
+        <v>196</v>
+      </c>
+      <c r="AR77" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS77" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT77">
+        <v>0.85</v>
+      </c>
+      <c r="AW77" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.76</v>
+      </c>
+    </row>
+    <row r="78" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I78" t="s">
         <v>266</v>
       </c>
@@ -7583,8 +8748,24 @@
       <c r="AN78" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="79" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ78" t="s">
+        <v>197</v>
+      </c>
+      <c r="AR78" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS78" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT78">
+        <v>0.94</v>
+      </c>
+      <c r="AW78" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.88</v>
+      </c>
+    </row>
+    <row r="79" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I79" t="s">
         <v>266</v>
       </c>
@@ -7651,8 +8832,24 @@
       <c r="AN79" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="80" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ79" t="s">
+        <v>198</v>
+      </c>
+      <c r="AR79" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS79" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT79">
+        <v>0.88</v>
+      </c>
+      <c r="AW79" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.73</v>
+      </c>
+    </row>
+    <row r="80" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I80" t="s">
         <v>266</v>
       </c>
@@ -7719,8 +8916,24 @@
       <c r="AN80" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="81" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ80" t="s">
+        <v>199</v>
+      </c>
+      <c r="AR80" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS80" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT80">
+        <v>0.94</v>
+      </c>
+      <c r="AW80" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.72</v>
+      </c>
+    </row>
+    <row r="81" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I81" t="s">
         <v>266</v>
       </c>
@@ -7787,8 +9000,24 @@
       <c r="AN81" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="82" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ81" t="s">
+        <v>200</v>
+      </c>
+      <c r="AR81" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS81" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT81">
+        <v>0.89</v>
+      </c>
+      <c r="AW81" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="82" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I82" t="s">
         <v>266</v>
       </c>
@@ -7855,8 +9084,24 @@
       <c r="AN82" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="83" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ82" t="s">
+        <v>201</v>
+      </c>
+      <c r="AR82" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS82" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT82">
+        <v>0.91</v>
+      </c>
+      <c r="AW82" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="83" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I83" t="s">
         <v>266</v>
       </c>
@@ -7923,8 +9168,24 @@
       <c r="AN83" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="84" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ83" t="s">
+        <v>202</v>
+      </c>
+      <c r="AR83" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS83" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT83">
+        <v>0.85</v>
+      </c>
+      <c r="AW83" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.77</v>
+      </c>
+    </row>
+    <row r="84" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I84" t="s">
         <v>266</v>
       </c>
@@ -7991,8 +9252,24 @@
       <c r="AN84" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="85" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ84" t="s">
+        <v>203</v>
+      </c>
+      <c r="AR84" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS84" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT84">
+        <v>0.81</v>
+      </c>
+      <c r="AW84" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="85" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I85" t="s">
         <v>266</v>
       </c>
@@ -8059,8 +9336,24 @@
       <c r="AN85" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="86" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ85" t="s">
+        <v>204</v>
+      </c>
+      <c r="AR85" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS85" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT85">
+        <v>0.93</v>
+      </c>
+      <c r="AW85" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.74</v>
+      </c>
+    </row>
+    <row r="86" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I86" t="s">
         <v>266</v>
       </c>
@@ -8127,8 +9420,24 @@
       <c r="AN86" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="87" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ86" t="s">
+        <v>205</v>
+      </c>
+      <c r="AR86" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS86" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT86">
+        <v>0.84</v>
+      </c>
+      <c r="AW86" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.71</v>
+      </c>
+    </row>
+    <row r="87" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I87" t="s">
         <v>266</v>
       </c>
@@ -8195,8 +9504,24 @@
       <c r="AN87" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="88" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ87" t="s">
+        <v>206</v>
+      </c>
+      <c r="AR87" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS87" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT87">
+        <v>0.8</v>
+      </c>
+      <c r="AW87" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.81</v>
+      </c>
+    </row>
+    <row r="88" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I88" t="s">
         <v>266</v>
       </c>
@@ -8263,8 +9588,24 @@
       <c r="AN88" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="89" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ88" t="s">
+        <v>207</v>
+      </c>
+      <c r="AR88" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS88" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT88">
+        <v>0.87</v>
+      </c>
+      <c r="AW88" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.86</v>
+      </c>
+    </row>
+    <row r="89" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I89" t="s">
         <v>266</v>
       </c>
@@ -8331,8 +9672,24 @@
       <c r="AN89" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="90" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ89" t="s">
+        <v>208</v>
+      </c>
+      <c r="AR89" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS89" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT89">
+        <v>0.75</v>
+      </c>
+      <c r="AW89" s="2">
+        <f t="shared" ca="1" si="1"/>
+        <v>0.82</v>
+      </c>
+    </row>
+    <row r="90" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I90" t="s">
         <v>266</v>
       </c>
@@ -8399,8 +9756,24 @@
       <c r="AN90" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="91" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ90" t="s">
+        <v>209</v>
+      </c>
+      <c r="AR90" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS90" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT90">
+        <v>0.94</v>
+      </c>
+      <c r="AW90" s="2">
+        <f t="shared" ref="AW90:AW98" ca="1" si="2">RANDBETWEEN(70,95)/100</f>
+        <v>0.82</v>
+      </c>
+    </row>
+    <row r="91" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I91" t="s">
         <v>266</v>
       </c>
@@ -8467,8 +9840,24 @@
       <c r="AN91" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="92" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ91" t="s">
+        <v>210</v>
+      </c>
+      <c r="AR91" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS91" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT91">
+        <v>0.8</v>
+      </c>
+      <c r="AW91" s="2">
+        <f t="shared" ca="1" si="2"/>
+        <v>0.76</v>
+      </c>
+    </row>
+    <row r="92" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I92" t="s">
         <v>266</v>
       </c>
@@ -8535,8 +9924,24 @@
       <c r="AN92" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="93" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ92" t="s">
+        <v>211</v>
+      </c>
+      <c r="AR92" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS92" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT92">
+        <v>0.7</v>
+      </c>
+      <c r="AW92" s="2">
+        <f t="shared" ca="1" si="2"/>
+        <v>0.84</v>
+      </c>
+    </row>
+    <row r="93" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I93" t="s">
         <v>266</v>
       </c>
@@ -8603,8 +10008,24 @@
       <c r="AN93" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="94" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ93" t="s">
+        <v>212</v>
+      </c>
+      <c r="AR93" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS93" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT93">
+        <v>0.82</v>
+      </c>
+      <c r="AW93" s="2">
+        <f t="shared" ca="1" si="2"/>
+        <v>0.92</v>
+      </c>
+    </row>
+    <row r="94" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I94" t="s">
         <v>266</v>
       </c>
@@ -8671,8 +10092,24 @@
       <c r="AN94" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="95" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ94" t="s">
+        <v>213</v>
+      </c>
+      <c r="AR94" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS94" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT94">
+        <v>0.95</v>
+      </c>
+      <c r="AW94" s="2">
+        <f t="shared" ca="1" si="2"/>
+        <v>0.82</v>
+      </c>
+    </row>
+    <row r="95" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I95" t="s">
         <v>266</v>
       </c>
@@ -8739,8 +10176,24 @@
       <c r="AN95" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="96" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ95" t="s">
+        <v>214</v>
+      </c>
+      <c r="AR95" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS95" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT95">
+        <v>0.76</v>
+      </c>
+      <c r="AW95" s="2">
+        <f t="shared" ca="1" si="2"/>
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="96" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I96" t="s">
         <v>266</v>
       </c>
@@ -8807,8 +10260,24 @@
       <c r="AN96" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="97" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ96" t="s">
+        <v>215</v>
+      </c>
+      <c r="AR96" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS96" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT96">
+        <v>0.93</v>
+      </c>
+      <c r="AW96" s="2">
+        <f t="shared" ca="1" si="2"/>
+        <v>0.89</v>
+      </c>
+    </row>
+    <row r="97" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I97" t="s">
         <v>266</v>
       </c>
@@ -8875,8 +10344,24 @@
       <c r="AN97" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="98" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ97" t="s">
+        <v>216</v>
+      </c>
+      <c r="AR97" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS97" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT97">
+        <v>0.89</v>
+      </c>
+      <c r="AW97" s="2">
+        <f t="shared" ca="1" si="2"/>
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="98" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I98" t="s">
         <v>266</v>
       </c>
@@ -8943,8 +10428,24 @@
       <c r="AN98" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="99" spans="9:40" x14ac:dyDescent="0.25">
+      <c r="AQ98" t="s">
+        <v>217</v>
+      </c>
+      <c r="AR98" t="s">
+        <v>286</v>
+      </c>
+      <c r="AS98" t="s">
+        <v>240</v>
+      </c>
+      <c r="AT98">
+        <v>0.79</v>
+      </c>
+      <c r="AW98" s="2">
+        <f t="shared" ca="1" si="2"/>
+        <v>0.93</v>
+      </c>
+    </row>
+    <row r="99" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I99" t="s">
         <v>267</v>
       </c>
@@ -8979,7 +10480,7 @@
         <v>1.7573439583804459E-2</v>
       </c>
     </row>
-    <row r="100" spans="9:40" x14ac:dyDescent="0.25">
+    <row r="100" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I100" t="s">
         <v>267</v>
       </c>
@@ -9014,7 +10515,7 @@
         <v>3.549030522775862E-3</v>
       </c>
     </row>
-    <row r="101" spans="9:40" x14ac:dyDescent="0.25">
+    <row r="101" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I101" t="s">
         <v>267</v>
       </c>
@@ -9049,7 +10550,7 @@
         <v>3.2008138253697617E-2</v>
       </c>
     </row>
-    <row r="102" spans="9:40" x14ac:dyDescent="0.25">
+    <row r="102" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I102" t="s">
         <v>267</v>
       </c>
@@ -9084,7 +10585,7 @@
         <v>3.5595926097493078E-3</v>
       </c>
     </row>
-    <row r="103" spans="9:40" x14ac:dyDescent="0.25">
+    <row r="103" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I103" t="s">
         <v>267</v>
       </c>
@@ -9119,7 +10620,7 @@
         <v>1.0678471251817045E-2</v>
       </c>
     </row>
-    <row r="104" spans="9:40" x14ac:dyDescent="0.25">
+    <row r="104" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I104" t="s">
         <v>267</v>
       </c>
@@ -9154,7 +10655,7 @@
         <v>3.5562894851714701E-3</v>
       </c>
     </row>
-    <row r="105" spans="9:40" x14ac:dyDescent="0.25">
+    <row r="105" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I105" t="s">
         <v>267</v>
       </c>
@@ -9189,7 +10690,7 @@
         <v>3.5440857255036491E-3</v>
       </c>
     </row>
-    <row r="106" spans="9:40" x14ac:dyDescent="0.25">
+    <row r="106" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I106" t="s">
         <v>267</v>
       </c>
@@ -9224,7 +10725,7 @@
         <v>1.0554198606771802E-2</v>
       </c>
     </row>
-    <row r="107" spans="9:40" x14ac:dyDescent="0.25">
+    <row r="107" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I107" t="s">
         <v>267</v>
       </c>
@@ -9259,7 +10760,7 @@
         <v>1.5916331913035826E-2</v>
       </c>
     </row>
-    <row r="108" spans="9:40" x14ac:dyDescent="0.25">
+    <row r="108" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I108" t="s">
         <v>267</v>
       </c>
@@ -9294,7 +10795,7 @@
         <v>3.2085184733168996E-3</v>
       </c>
     </row>
-    <row r="109" spans="9:40" x14ac:dyDescent="0.25">
+    <row r="109" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I109" t="s">
         <v>267</v>
       </c>
@@ -9329,7 +10830,7 @@
         <v>2.8854869593476187E-2</v>
       </c>
     </row>
-    <row r="110" spans="9:40" x14ac:dyDescent="0.25">
+    <row r="110" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I110" t="s">
         <v>267</v>
       </c>
@@ -9364,7 +10865,7 @@
         <v>3.2092305241240983E-3</v>
       </c>
     </row>
-    <row r="111" spans="9:40" x14ac:dyDescent="0.25">
+    <row r="111" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I111" t="s">
         <v>267</v>
       </c>
@@ -9399,7 +10900,7 @@
         <v>9.6277410203450178E-3</v>
       </c>
     </row>
-    <row r="112" spans="9:40" x14ac:dyDescent="0.25">
+    <row r="112" spans="9:49" x14ac:dyDescent="0.25">
       <c r="I112" t="s">
         <v>267</v>
       </c>

</xml_diff>

<commit_message>
Remvoing COM_PEAK and com_pkflx from Scen_bau.xlsx
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_bau.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_bau.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89DAFF1C-AEF9-4E69-ABFD-A2D1EFC4DC10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A92FB753-D999-4695-BC19-F7F163A1C2CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Demand" sheetId="1" r:id="rId1"/>
@@ -25,6 +25,7 @@
     <externalReference r:id="rId8"/>
   </externalReferences>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -73,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8003" uniqueCount="285">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8003" uniqueCount="286">
   <si>
     <t>~TFM_INS-TS</t>
   </si>
@@ -929,6 +930,9 @@
   <si>
     <t>elc</t>
   </si>
+  <si>
+    <t>TFM_DINS-AT</t>
+  </si>
 </sst>
 </file>
 
@@ -1089,7 +1093,7 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1116,7 +1120,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="9" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="9"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="9" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="10">
     <cellStyle name="Comma 2" xfId="3" xr:uid="{45765176-8E4D-467C-8B17-17A7F0C6EBE1}"/>
@@ -1488,7 +1491,34 @@
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
+      <c r="E3" s="7">
+        <f>SUM(E5:E8)</f>
+        <v>8.4914999999999985</v>
+      </c>
+      <c r="F3" s="7">
+        <f t="shared" ref="F3:K3" si="0">SUM(F5:F8)</f>
+        <v>8.4719999999999995</v>
+      </c>
+      <c r="G3" s="7">
+        <f t="shared" si="0"/>
+        <v>9.109</v>
+      </c>
+      <c r="H3" s="7">
+        <f t="shared" si="0"/>
+        <v>10.274000000000001</v>
+      </c>
+      <c r="I3" s="7">
+        <f t="shared" si="0"/>
+        <v>11.359</v>
+      </c>
+      <c r="J3" s="7">
+        <f t="shared" si="0"/>
+        <v>12.954000000000001</v>
+      </c>
+      <c r="K3" s="7">
+        <f t="shared" si="0"/>
+        <v>14.578999999999999</v>
+      </c>
       <c r="O3" t="s">
         <v>34</v>
       </c>
@@ -1883,14 +1913,14 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B20" t="s">
+    <row r="24" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B24" t="s">
         <v>283</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C24" t="s">
         <v>284</v>
       </c>
-      <c r="E20">
+      <c r="E24">
         <v>1</v>
       </c>
     </row>
@@ -1948,8 +1978,8 @@
       <c r="X1" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="AB1" s="20" t="s">
-        <v>49</v>
+      <c r="AB1" s="11" t="s">
+        <v>285</v>
       </c>
       <c r="AF1" s="11" t="s">
         <v>67</v>
@@ -4380,7 +4410,7 @@
       </c>
       <c r="AX25" s="2">
         <f ca="1">RANDBETWEEN(70,95)/100</f>
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="26" spans="9:50" x14ac:dyDescent="0.25">
@@ -4479,7 +4509,7 @@
       </c>
       <c r="AX26" s="2">
         <f t="shared" ref="AX26:AX89" ca="1" si="1">RANDBETWEEN(70,95)/100</f>
-        <v>0.82</v>
+        <v>0.74</v>
       </c>
     </row>
     <row r="27" spans="9:50" x14ac:dyDescent="0.25">
@@ -4578,7 +4608,7 @@
       </c>
       <c r="AX27" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.74</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="28" spans="9:50" x14ac:dyDescent="0.25">
@@ -4677,7 +4707,7 @@
       </c>
       <c r="AX28" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.73</v>
+        <v>0.88</v>
       </c>
     </row>
     <row r="29" spans="9:50" x14ac:dyDescent="0.25">
@@ -4776,7 +4806,7 @@
       </c>
       <c r="AX29" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.75</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="30" spans="9:50" x14ac:dyDescent="0.25">
@@ -4875,7 +4905,7 @@
       </c>
       <c r="AX30" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.89</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="31" spans="9:50" x14ac:dyDescent="0.25">
@@ -4974,7 +5004,7 @@
       </c>
       <c r="AX31" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.83</v>
+        <v>0.91</v>
       </c>
     </row>
     <row r="32" spans="9:50" x14ac:dyDescent="0.25">
@@ -5073,7 +5103,7 @@
       </c>
       <c r="AX32" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.78</v>
+        <v>0.89</v>
       </c>
     </row>
     <row r="33" spans="9:50" x14ac:dyDescent="0.25">
@@ -5172,7 +5202,7 @@
       </c>
       <c r="AX33" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="34" spans="9:50" x14ac:dyDescent="0.25">
@@ -5271,7 +5301,7 @@
       </c>
       <c r="AX34" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.88</v>
+        <v>0.91</v>
       </c>
     </row>
     <row r="35" spans="9:50" x14ac:dyDescent="0.25">
@@ -5370,7 +5400,7 @@
       </c>
       <c r="AX35" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.77</v>
+        <v>0.74</v>
       </c>
     </row>
     <row r="36" spans="9:50" x14ac:dyDescent="0.25">
@@ -5469,7 +5499,7 @@
       </c>
       <c r="AX36" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.94</v>
+        <v>0.88</v>
       </c>
     </row>
     <row r="37" spans="9:50" x14ac:dyDescent="0.25">
@@ -5667,7 +5697,7 @@
       </c>
       <c r="AX38" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.71</v>
+        <v>0.92</v>
       </c>
     </row>
     <row r="39" spans="9:50" x14ac:dyDescent="0.25">
@@ -5754,7 +5784,7 @@
       </c>
       <c r="AX39" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.73</v>
+        <v>0.74</v>
       </c>
     </row>
     <row r="40" spans="9:50" x14ac:dyDescent="0.25">
@@ -5841,7 +5871,7 @@
       </c>
       <c r="AX40" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.84</v>
+        <v>0.87</v>
       </c>
     </row>
     <row r="41" spans="9:50" x14ac:dyDescent="0.25">
@@ -6015,7 +6045,7 @@
       </c>
       <c r="AX42" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.82</v>
+        <v>0.94</v>
       </c>
     </row>
     <row r="43" spans="9:50" x14ac:dyDescent="0.25">
@@ -6102,7 +6132,7 @@
       </c>
       <c r="AX43" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.73</v>
+        <v>0.88</v>
       </c>
     </row>
     <row r="44" spans="9:50" x14ac:dyDescent="0.25">
@@ -6189,7 +6219,7 @@
       </c>
       <c r="AX44" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.91</v>
+        <v>0.89</v>
       </c>
     </row>
     <row r="45" spans="9:50" x14ac:dyDescent="0.25">
@@ -6276,7 +6306,7 @@
       </c>
       <c r="AX45" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.91</v>
+        <v>0.74</v>
       </c>
     </row>
     <row r="46" spans="9:50" x14ac:dyDescent="0.25">
@@ -6363,7 +6393,7 @@
       </c>
       <c r="AX46" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.94</v>
+        <v>0.79</v>
       </c>
     </row>
     <row r="47" spans="9:50" x14ac:dyDescent="0.25">
@@ -6450,7 +6480,7 @@
       </c>
       <c r="AX47" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.9</v>
+        <v>0.84</v>
       </c>
     </row>
     <row r="48" spans="9:50" x14ac:dyDescent="0.25">
@@ -6537,7 +6567,7 @@
       </c>
       <c r="AX48" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.72</v>
+        <v>0.93</v>
       </c>
     </row>
     <row r="49" spans="9:50" x14ac:dyDescent="0.25">
@@ -6624,7 +6654,7 @@
       </c>
       <c r="AX49" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.88</v>
+        <v>0.72</v>
       </c>
     </row>
     <row r="50" spans="9:50" x14ac:dyDescent="0.25">
@@ -6711,7 +6741,7 @@
       </c>
       <c r="AX50" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.73</v>
+        <v>0.89</v>
       </c>
     </row>
     <row r="51" spans="9:50" x14ac:dyDescent="0.25">
@@ -6798,7 +6828,7 @@
       </c>
       <c r="AX51" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.72</v>
+        <v>0.89</v>
       </c>
     </row>
     <row r="52" spans="9:50" x14ac:dyDescent="0.25">
@@ -6885,7 +6915,7 @@
       </c>
       <c r="AX52" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.86</v>
+        <v>0.89</v>
       </c>
     </row>
     <row r="53" spans="9:50" x14ac:dyDescent="0.25">
@@ -6972,7 +7002,7 @@
       </c>
       <c r="AX53" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.93</v>
+        <v>0.88</v>
       </c>
     </row>
     <row r="54" spans="9:50" x14ac:dyDescent="0.25">
@@ -7059,7 +7089,7 @@
       </c>
       <c r="AX54" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.92</v>
+        <v>0.76</v>
       </c>
     </row>
     <row r="55" spans="9:50" x14ac:dyDescent="0.25">
@@ -7146,7 +7176,7 @@
       </c>
       <c r="AX55" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.73</v>
+        <v>0.76</v>
       </c>
     </row>
     <row r="56" spans="9:50" x14ac:dyDescent="0.25">
@@ -7233,7 +7263,7 @@
       </c>
       <c r="AX56" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.76</v>
+        <v>0.77</v>
       </c>
     </row>
     <row r="57" spans="9:50" x14ac:dyDescent="0.25">
@@ -7320,7 +7350,7 @@
       </c>
       <c r="AX57" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.73</v>
+        <v>0.82</v>
       </c>
     </row>
     <row r="58" spans="9:50" x14ac:dyDescent="0.25">
@@ -7407,7 +7437,7 @@
       </c>
       <c r="AX58" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.95</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="59" spans="9:50" x14ac:dyDescent="0.25">
@@ -7494,7 +7524,7 @@
       </c>
       <c r="AX59" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.86</v>
+        <v>0.78</v>
       </c>
     </row>
     <row r="60" spans="9:50" x14ac:dyDescent="0.25">
@@ -7581,7 +7611,7 @@
       </c>
       <c r="AX60" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.8</v>
+        <v>0.77</v>
       </c>
     </row>
     <row r="61" spans="9:50" x14ac:dyDescent="0.25">
@@ -7668,7 +7698,7 @@
       </c>
       <c r="AX61" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.77</v>
+        <v>0.76</v>
       </c>
     </row>
     <row r="62" spans="9:50" x14ac:dyDescent="0.25">
@@ -7755,7 +7785,7 @@
       </c>
       <c r="AX62" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.94</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="63" spans="9:50" x14ac:dyDescent="0.25">
@@ -7842,7 +7872,7 @@
       </c>
       <c r="AX63" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.86</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="64" spans="9:50" x14ac:dyDescent="0.25">
@@ -8016,7 +8046,7 @@
       </c>
       <c r="AX65" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.9</v>
+        <v>0.72</v>
       </c>
     </row>
     <row r="66" spans="9:50" x14ac:dyDescent="0.25">
@@ -8103,7 +8133,7 @@
       </c>
       <c r="AX66" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.83</v>
+        <v>0.91</v>
       </c>
     </row>
     <row r="67" spans="9:50" x14ac:dyDescent="0.25">
@@ -8190,7 +8220,7 @@
       </c>
       <c r="AX67" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.8</v>
+        <v>0.91</v>
       </c>
     </row>
     <row r="68" spans="9:50" x14ac:dyDescent="0.25">
@@ -8277,7 +8307,7 @@
       </c>
       <c r="AX68" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.85</v>
+        <v>0.74</v>
       </c>
     </row>
     <row r="69" spans="9:50" x14ac:dyDescent="0.25">
@@ -8364,7 +8394,7 @@
       </c>
       <c r="AX69" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.8</v>
+        <v>0.79</v>
       </c>
     </row>
     <row r="70" spans="9:50" x14ac:dyDescent="0.25">
@@ -8451,7 +8481,7 @@
       </c>
       <c r="AX70" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.84</v>
+        <v>0.94</v>
       </c>
     </row>
     <row r="71" spans="9:50" x14ac:dyDescent="0.25">
@@ -8538,7 +8568,7 @@
       </c>
       <c r="AX71" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.9</v>
+        <v>0.71</v>
       </c>
     </row>
     <row r="72" spans="9:50" x14ac:dyDescent="0.25">
@@ -8625,7 +8655,7 @@
       </c>
       <c r="AX72" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.75</v>
+        <v>0.77</v>
       </c>
     </row>
     <row r="73" spans="9:50" x14ac:dyDescent="0.25">
@@ -8712,7 +8742,7 @@
       </c>
       <c r="AX73" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.74</v>
+        <v>0.88</v>
       </c>
     </row>
     <row r="74" spans="9:50" x14ac:dyDescent="0.25">
@@ -8799,7 +8829,7 @@
       </c>
       <c r="AX74" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.81</v>
+        <v>0.88</v>
       </c>
     </row>
     <row r="75" spans="9:50" x14ac:dyDescent="0.25">
@@ -8886,7 +8916,7 @@
       </c>
       <c r="AX75" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.94</v>
+        <v>0.81</v>
       </c>
     </row>
     <row r="76" spans="9:50" x14ac:dyDescent="0.25">
@@ -8973,7 +9003,7 @@
       </c>
       <c r="AX76" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.77</v>
+        <v>0.89</v>
       </c>
     </row>
     <row r="77" spans="9:50" x14ac:dyDescent="0.25">
@@ -9060,7 +9090,7 @@
       </c>
       <c r="AX77" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.82</v>
+        <v>0.91</v>
       </c>
     </row>
     <row r="78" spans="9:50" x14ac:dyDescent="0.25">
@@ -9147,7 +9177,7 @@
       </c>
       <c r="AX78" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.93</v>
+        <v>0.76</v>
       </c>
     </row>
     <row r="79" spans="9:50" x14ac:dyDescent="0.25">
@@ -9234,7 +9264,7 @@
       </c>
       <c r="AX79" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.94</v>
+        <v>0.74</v>
       </c>
     </row>
     <row r="80" spans="9:50" x14ac:dyDescent="0.25">
@@ -9321,7 +9351,7 @@
       </c>
       <c r="AX80" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
     </row>
     <row r="81" spans="9:50" x14ac:dyDescent="0.25">
@@ -9408,7 +9438,7 @@
       </c>
       <c r="AX81" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.75</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="82" spans="9:50" x14ac:dyDescent="0.25">
@@ -9495,7 +9525,7 @@
       </c>
       <c r="AX82" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.95</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="83" spans="9:50" x14ac:dyDescent="0.25">
@@ -9582,7 +9612,7 @@
       </c>
       <c r="AX83" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.84</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="84" spans="9:50" x14ac:dyDescent="0.25">
@@ -9669,7 +9699,7 @@
       </c>
       <c r="AX84" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.78</v>
+        <v>0.94</v>
       </c>
     </row>
     <row r="85" spans="9:50" x14ac:dyDescent="0.25">
@@ -9756,7 +9786,7 @@
       </c>
       <c r="AX85" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.79</v>
+        <v>0.94</v>
       </c>
     </row>
     <row r="86" spans="9:50" x14ac:dyDescent="0.25">
@@ -9843,7 +9873,7 @@
       </c>
       <c r="AX86" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.7</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="87" spans="9:50" x14ac:dyDescent="0.25">
@@ -9930,7 +9960,7 @@
       </c>
       <c r="AX87" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.91</v>
+        <v>0.88</v>
       </c>
     </row>
     <row r="88" spans="9:50" x14ac:dyDescent="0.25">
@@ -10017,7 +10047,7 @@
       </c>
       <c r="AX88" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.81</v>
+        <v>0.73</v>
       </c>
     </row>
     <row r="89" spans="9:50" x14ac:dyDescent="0.25">
@@ -10104,7 +10134,7 @@
       </c>
       <c r="AX89" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.87</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="90" spans="9:50" x14ac:dyDescent="0.25">
@@ -10191,7 +10221,7 @@
       </c>
       <c r="AX90" s="2">
         <f t="shared" ref="AX90:AX98" ca="1" si="2">RANDBETWEEN(70,95)/100</f>
-        <v>0.81</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="91" spans="9:50" x14ac:dyDescent="0.25">
@@ -10278,7 +10308,7 @@
       </c>
       <c r="AX91" s="2">
         <f t="shared" ca="1" si="2"/>
-        <v>0.86</v>
+        <v>0.78</v>
       </c>
     </row>
     <row r="92" spans="9:50" x14ac:dyDescent="0.25">
@@ -10365,7 +10395,7 @@
       </c>
       <c r="AX92" s="2">
         <f t="shared" ca="1" si="2"/>
-        <v>0.77</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="93" spans="9:50" x14ac:dyDescent="0.25">
@@ -10452,7 +10482,7 @@
       </c>
       <c r="AX93" s="2">
         <f t="shared" ca="1" si="2"/>
-        <v>0.92</v>
+        <v>0.71</v>
       </c>
     </row>
     <row r="94" spans="9:50" x14ac:dyDescent="0.25">
@@ -10539,7 +10569,7 @@
       </c>
       <c r="AX94" s="2">
         <f t="shared" ca="1" si="2"/>
-        <v>0.77</v>
+        <v>0.74</v>
       </c>
     </row>
     <row r="95" spans="9:50" x14ac:dyDescent="0.25">
@@ -10626,7 +10656,7 @@
       </c>
       <c r="AX95" s="2">
         <f t="shared" ca="1" si="2"/>
-        <v>0.75</v>
+        <v>0.84</v>
       </c>
     </row>
     <row r="96" spans="9:50" x14ac:dyDescent="0.25">
@@ -10713,7 +10743,7 @@
       </c>
       <c r="AX96" s="2">
         <f t="shared" ca="1" si="2"/>
-        <v>0.8</v>
+        <v>0.77</v>
       </c>
     </row>
     <row r="97" spans="9:50" x14ac:dyDescent="0.25">
@@ -10800,7 +10830,7 @@
       </c>
       <c r="AX97" s="2">
         <f t="shared" ca="1" si="2"/>
-        <v>0.87</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="98" spans="9:50" x14ac:dyDescent="0.25">
@@ -10887,7 +10917,7 @@
       </c>
       <c r="AX98" s="2">
         <f t="shared" ca="1" si="2"/>
-        <v>0.85</v>
+        <v>0.78</v>
       </c>
     </row>
     <row r="99" spans="9:50" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
adding back COM_PEAK and COM_PKFLX to ELC
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_bau.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_bau.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A92FB753-D999-4695-BC19-F7F163A1C2CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D983772C-869C-4C52-AF2C-AFB1FDF277D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8003" uniqueCount="286">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8003" uniqueCount="285">
   <si>
     <t>~TFM_INS-TS</t>
   </si>
@@ -930,9 +930,6 @@
   <si>
     <t>elc</t>
   </si>
-  <si>
-    <t>TFM_DINS-AT</t>
-  </si>
 </sst>
 </file>
 
@@ -1913,14 +1910,14 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="2:16" x14ac:dyDescent="0.25">
-      <c r="B24" t="s">
+    <row r="20" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B20" t="s">
         <v>283</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C20" t="s">
         <v>284</v>
       </c>
-      <c r="E24">
+      <c r="E20">
         <v>1</v>
       </c>
     </row>
@@ -1979,7 +1976,7 @@
         <v>49</v>
       </c>
       <c r="AB1" s="11" t="s">
-        <v>285</v>
+        <v>49</v>
       </c>
       <c r="AF1" s="11" t="s">
         <v>67</v>
@@ -4608,7 +4605,7 @@
       </c>
       <c r="AX27" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.75</v>
+        <v>0.78</v>
       </c>
     </row>
     <row r="28" spans="9:50" x14ac:dyDescent="0.25">
@@ -4707,7 +4704,7 @@
       </c>
       <c r="AX28" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.88</v>
+        <v>0.74</v>
       </c>
     </row>
     <row r="29" spans="9:50" x14ac:dyDescent="0.25">
@@ -4806,7 +4803,7 @@
       </c>
       <c r="AX29" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.8</v>
+        <v>0.92</v>
       </c>
     </row>
     <row r="30" spans="9:50" x14ac:dyDescent="0.25">
@@ -4905,7 +4902,7 @@
       </c>
       <c r="AX30" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.75</v>
+        <v>0.93</v>
       </c>
     </row>
     <row r="31" spans="9:50" x14ac:dyDescent="0.25">
@@ -5004,7 +5001,7 @@
       </c>
       <c r="AX31" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.91</v>
+        <v>0.92</v>
       </c>
     </row>
     <row r="32" spans="9:50" x14ac:dyDescent="0.25">
@@ -5103,7 +5100,7 @@
       </c>
       <c r="AX32" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.89</v>
+        <v>0.73</v>
       </c>
     </row>
     <row r="33" spans="9:50" x14ac:dyDescent="0.25">
@@ -5202,7 +5199,7 @@
       </c>
       <c r="AX33" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.8</v>
+        <v>0.91</v>
       </c>
     </row>
     <row r="34" spans="9:50" x14ac:dyDescent="0.25">
@@ -5301,7 +5298,7 @@
       </c>
       <c r="AX34" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.91</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="35" spans="9:50" x14ac:dyDescent="0.25">
@@ -5400,7 +5397,7 @@
       </c>
       <c r="AX35" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.74</v>
+        <v>0.94</v>
       </c>
     </row>
     <row r="36" spans="9:50" x14ac:dyDescent="0.25">
@@ -5499,7 +5496,7 @@
       </c>
       <c r="AX36" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.88</v>
+        <v>0.91</v>
       </c>
     </row>
     <row r="37" spans="9:50" x14ac:dyDescent="0.25">
@@ -5598,7 +5595,7 @@
       </c>
       <c r="AX37" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.93</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="38" spans="9:50" x14ac:dyDescent="0.25">
@@ -5697,7 +5694,7 @@
       </c>
       <c r="AX38" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.92</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="39" spans="9:50" x14ac:dyDescent="0.25">
@@ -5784,7 +5781,7 @@
       </c>
       <c r="AX39" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.74</v>
+        <v>0.83</v>
       </c>
     </row>
     <row r="40" spans="9:50" x14ac:dyDescent="0.25">
@@ -5871,7 +5868,7 @@
       </c>
       <c r="AX40" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.87</v>
+        <v>0.83</v>
       </c>
     </row>
     <row r="41" spans="9:50" x14ac:dyDescent="0.25">
@@ -5958,7 +5955,7 @@
       </c>
       <c r="AX41" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.8</v>
+        <v>0.87</v>
       </c>
     </row>
     <row r="42" spans="9:50" x14ac:dyDescent="0.25">
@@ -6045,7 +6042,7 @@
       </c>
       <c r="AX42" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.94</v>
+        <v>0.82</v>
       </c>
     </row>
     <row r="43" spans="9:50" x14ac:dyDescent="0.25">
@@ -6132,7 +6129,7 @@
       </c>
       <c r="AX43" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.88</v>
+        <v>0.74</v>
       </c>
     </row>
     <row r="44" spans="9:50" x14ac:dyDescent="0.25">
@@ -6219,7 +6216,7 @@
       </c>
       <c r="AX44" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.89</v>
+        <v>0.76</v>
       </c>
     </row>
     <row r="45" spans="9:50" x14ac:dyDescent="0.25">
@@ -6306,7 +6303,7 @@
       </c>
       <c r="AX45" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.74</v>
+        <v>0.82</v>
       </c>
     </row>
     <row r="46" spans="9:50" x14ac:dyDescent="0.25">
@@ -6393,7 +6390,7 @@
       </c>
       <c r="AX46" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.79</v>
+        <v>0.82</v>
       </c>
     </row>
     <row r="47" spans="9:50" x14ac:dyDescent="0.25">
@@ -6480,7 +6477,7 @@
       </c>
       <c r="AX47" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.84</v>
+        <v>0.79</v>
       </c>
     </row>
     <row r="48" spans="9:50" x14ac:dyDescent="0.25">
@@ -6567,7 +6564,7 @@
       </c>
       <c r="AX48" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.93</v>
+        <v>0.82</v>
       </c>
     </row>
     <row r="49" spans="9:50" x14ac:dyDescent="0.25">
@@ -6654,7 +6651,7 @@
       </c>
       <c r="AX49" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.72</v>
+        <v>0.87</v>
       </c>
     </row>
     <row r="50" spans="9:50" x14ac:dyDescent="0.25">
@@ -6741,7 +6738,7 @@
       </c>
       <c r="AX50" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.89</v>
+        <v>0.74</v>
       </c>
     </row>
     <row r="51" spans="9:50" x14ac:dyDescent="0.25">
@@ -6828,7 +6825,7 @@
       </c>
       <c r="AX51" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.89</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="52" spans="9:50" x14ac:dyDescent="0.25">
@@ -6915,7 +6912,7 @@
       </c>
       <c r="AX52" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.89</v>
+        <v>0.78</v>
       </c>
     </row>
     <row r="53" spans="9:50" x14ac:dyDescent="0.25">
@@ -7002,7 +6999,7 @@
       </c>
       <c r="AX53" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.88</v>
+        <v>0.79</v>
       </c>
     </row>
     <row r="54" spans="9:50" x14ac:dyDescent="0.25">
@@ -7089,7 +7086,7 @@
       </c>
       <c r="AX54" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.76</v>
+        <v>0.84</v>
       </c>
     </row>
     <row r="55" spans="9:50" x14ac:dyDescent="0.25">
@@ -7176,7 +7173,7 @@
       </c>
       <c r="AX55" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.76</v>
+        <v>0.91</v>
       </c>
     </row>
     <row r="56" spans="9:50" x14ac:dyDescent="0.25">
@@ -7263,7 +7260,7 @@
       </c>
       <c r="AX56" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.77</v>
+        <v>0.71</v>
       </c>
     </row>
     <row r="57" spans="9:50" x14ac:dyDescent="0.25">
@@ -7350,7 +7347,7 @@
       </c>
       <c r="AX57" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.82</v>
+        <v>0.73</v>
       </c>
     </row>
     <row r="58" spans="9:50" x14ac:dyDescent="0.25">
@@ -7437,7 +7434,7 @@
       </c>
       <c r="AX58" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.85</v>
+        <v>0.89</v>
       </c>
     </row>
     <row r="59" spans="9:50" x14ac:dyDescent="0.25">
@@ -7524,7 +7521,7 @@
       </c>
       <c r="AX59" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.78</v>
+        <v>0.77</v>
       </c>
     </row>
     <row r="60" spans="9:50" x14ac:dyDescent="0.25">
@@ -7611,7 +7608,7 @@
       </c>
       <c r="AX60" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.77</v>
+        <v>0.86</v>
       </c>
     </row>
     <row r="61" spans="9:50" x14ac:dyDescent="0.25">
@@ -7785,7 +7782,7 @@
       </c>
       <c r="AX62" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="63" spans="9:50" x14ac:dyDescent="0.25">
@@ -7872,7 +7869,7 @@
       </c>
       <c r="AX63" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.8</v>
+        <v>0.93</v>
       </c>
     </row>
     <row r="64" spans="9:50" x14ac:dyDescent="0.25">
@@ -7959,7 +7956,7 @@
       </c>
       <c r="AX64" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.71</v>
+        <v>0.84</v>
       </c>
     </row>
     <row r="65" spans="9:50" x14ac:dyDescent="0.25">
@@ -8046,7 +8043,7 @@
       </c>
       <c r="AX65" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.72</v>
+        <v>0.92</v>
       </c>
     </row>
     <row r="66" spans="9:50" x14ac:dyDescent="0.25">
@@ -8133,7 +8130,7 @@
       </c>
       <c r="AX66" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.91</v>
+        <v>0.78</v>
       </c>
     </row>
     <row r="67" spans="9:50" x14ac:dyDescent="0.25">
@@ -8220,7 +8217,7 @@
       </c>
       <c r="AX67" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.91</v>
+        <v>0.79</v>
       </c>
     </row>
     <row r="68" spans="9:50" x14ac:dyDescent="0.25">
@@ -8307,7 +8304,7 @@
       </c>
       <c r="AX68" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.74</v>
+        <v>0.87</v>
       </c>
     </row>
     <row r="69" spans="9:50" x14ac:dyDescent="0.25">
@@ -8394,7 +8391,7 @@
       </c>
       <c r="AX69" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.79</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="70" spans="9:50" x14ac:dyDescent="0.25">
@@ -8481,7 +8478,7 @@
       </c>
       <c r="AX70" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.94</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="71" spans="9:50" x14ac:dyDescent="0.25">
@@ -8568,7 +8565,7 @@
       </c>
       <c r="AX71" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.71</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="72" spans="9:50" x14ac:dyDescent="0.25">
@@ -8655,7 +8652,7 @@
       </c>
       <c r="AX72" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.77</v>
+        <v>0.92</v>
       </c>
     </row>
     <row r="73" spans="9:50" x14ac:dyDescent="0.25">
@@ -8742,7 +8739,7 @@
       </c>
       <c r="AX73" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.88</v>
+        <v>0.79</v>
       </c>
     </row>
     <row r="74" spans="9:50" x14ac:dyDescent="0.25">
@@ -8829,7 +8826,7 @@
       </c>
       <c r="AX74" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.88</v>
+        <v>0.82</v>
       </c>
     </row>
     <row r="75" spans="9:50" x14ac:dyDescent="0.25">
@@ -8916,7 +8913,7 @@
       </c>
       <c r="AX75" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.81</v>
+        <v>0.93</v>
       </c>
     </row>
     <row r="76" spans="9:50" x14ac:dyDescent="0.25">
@@ -9003,7 +9000,7 @@
       </c>
       <c r="AX76" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.89</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="77" spans="9:50" x14ac:dyDescent="0.25">
@@ -9090,7 +9087,7 @@
       </c>
       <c r="AX77" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.91</v>
+        <v>0.71</v>
       </c>
     </row>
     <row r="78" spans="9:50" x14ac:dyDescent="0.25">
@@ -9177,7 +9174,7 @@
       </c>
       <c r="AX78" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.76</v>
+        <v>0.79</v>
       </c>
     </row>
     <row r="79" spans="9:50" x14ac:dyDescent="0.25">
@@ -9264,7 +9261,7 @@
       </c>
       <c r="AX79" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.74</v>
+        <v>0.73</v>
       </c>
     </row>
     <row r="80" spans="9:50" x14ac:dyDescent="0.25">
@@ -9351,7 +9348,7 @@
       </c>
       <c r="AX80" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.86</v>
+        <v>0.77</v>
       </c>
     </row>
     <row r="81" spans="9:50" x14ac:dyDescent="0.25">
@@ -9438,7 +9435,7 @@
       </c>
       <c r="AX81" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.85</v>
+        <v>0.72</v>
       </c>
     </row>
     <row r="82" spans="9:50" x14ac:dyDescent="0.25">
@@ -9525,7 +9522,7 @@
       </c>
       <c r="AX82" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
     </row>
     <row r="83" spans="9:50" x14ac:dyDescent="0.25">
@@ -9612,7 +9609,7 @@
       </c>
       <c r="AX83" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
     </row>
     <row r="84" spans="9:50" x14ac:dyDescent="0.25">
@@ -9699,7 +9696,7 @@
       </c>
       <c r="AX84" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.94</v>
+        <v>0.81</v>
       </c>
     </row>
     <row r="85" spans="9:50" x14ac:dyDescent="0.25">
@@ -9786,7 +9783,7 @@
       </c>
       <c r="AX85" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.94</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="86" spans="9:50" x14ac:dyDescent="0.25">
@@ -9873,7 +9870,7 @@
       </c>
       <c r="AX86" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.75</v>
+        <v>0.86</v>
       </c>
     </row>
     <row r="87" spans="9:50" x14ac:dyDescent="0.25">
@@ -9960,7 +9957,7 @@
       </c>
       <c r="AX87" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.88</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="88" spans="9:50" x14ac:dyDescent="0.25">
@@ -10047,7 +10044,7 @@
       </c>
       <c r="AX88" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.73</v>
+        <v>0.71</v>
       </c>
     </row>
     <row r="89" spans="9:50" x14ac:dyDescent="0.25">
@@ -10134,7 +10131,7 @@
       </c>
       <c r="AX89" s="2">
         <f t="shared" ca="1" si="1"/>
-        <v>0.85</v>
+        <v>0.79</v>
       </c>
     </row>
     <row r="90" spans="9:50" x14ac:dyDescent="0.25">
@@ -10221,7 +10218,7 @@
       </c>
       <c r="AX90" s="2">
         <f t="shared" ref="AX90:AX98" ca="1" si="2">RANDBETWEEN(70,95)/100</f>
-        <v>0.95</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="91" spans="9:50" x14ac:dyDescent="0.25">
@@ -10308,7 +10305,7 @@
       </c>
       <c r="AX91" s="2">
         <f t="shared" ca="1" si="2"/>
-        <v>0.78</v>
+        <v>0.74</v>
       </c>
     </row>
     <row r="92" spans="9:50" x14ac:dyDescent="0.25">
@@ -10395,7 +10392,7 @@
       </c>
       <c r="AX92" s="2">
         <f t="shared" ca="1" si="2"/>
-        <v>0.9</v>
+        <v>0.88</v>
       </c>
     </row>
     <row r="93" spans="9:50" x14ac:dyDescent="0.25">
@@ -10482,7 +10479,7 @@
       </c>
       <c r="AX93" s="2">
         <f t="shared" ca="1" si="2"/>
-        <v>0.71</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="94" spans="9:50" x14ac:dyDescent="0.25">
@@ -10569,7 +10566,7 @@
       </c>
       <c r="AX94" s="2">
         <f t="shared" ca="1" si="2"/>
-        <v>0.74</v>
+        <v>0.76</v>
       </c>
     </row>
     <row r="95" spans="9:50" x14ac:dyDescent="0.25">
@@ -10656,7 +10653,7 @@
       </c>
       <c r="AX95" s="2">
         <f t="shared" ca="1" si="2"/>
-        <v>0.84</v>
+        <v>0.82</v>
       </c>
     </row>
     <row r="96" spans="9:50" x14ac:dyDescent="0.25">
@@ -10743,7 +10740,7 @@
       </c>
       <c r="AX96" s="2">
         <f t="shared" ca="1" si="2"/>
-        <v>0.77</v>
+        <v>0.74</v>
       </c>
     </row>
     <row r="97" spans="9:50" x14ac:dyDescent="0.25">
@@ -10830,7 +10827,7 @@
       </c>
       <c r="AX97" s="2">
         <f t="shared" ca="1" si="2"/>
-        <v>0.7</v>
+        <v>0.74</v>
       </c>
     </row>
     <row r="98" spans="9:50" x14ac:dyDescent="0.25">
@@ -10917,7 +10914,7 @@
       </c>
       <c r="AX98" s="2">
         <f t="shared" ca="1" si="2"/>
-        <v>0.78</v>
+        <v>0.89</v>
       </c>
     </row>
     <row r="99" spans="9:50" x14ac:dyDescent="0.25">

</xml_diff>